<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-08 16:35
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 16:11</t>
+          <t>2026-05-08 16:35</t>
         </is>
       </c>
     </row>
@@ -18297,9 +18297,9 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -18321,17 +18321,17 @@
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Downtime_0_trip_baht</t>
+          <t>Downtime_50_baht</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Downtime_1_trip_baht</t>
+          <t>Downtime_100_baht</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Blank_run_baht</t>
+          <t>Blank_run_50_baht</t>
         </is>
       </c>
       <c r="G1" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-08 17:40
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -135,10 +135,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 16:35</t>
+          <t>2026-05-08 17:39</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01–2026-05-31=6,500 @31.00-31.99, step 1.50%/฿ / 2026-04-12–2026-04-15=8,000 @50.00-50.99, step 1.50%/฿, floor 6,500 / 2026-04-01–2026-04-30=7,500 @50.00-50.99, step 1.50%/฿, floor 6,500 / ปกติ=7,500 @50.00-50.99, step 1.50%/฿</t>
+          <t>2026-05-01–2026-05-31=6,500.00 @31.00-31.99, step 1.50%/฿ / 2026-04-12–2026-04-15=8,000.00 @50.00-50.99, step 1.50%/฿, floor 6,500.00 / 2026-04-01–2026-04-30=7,500.00 @50.00-50.99, step 1.50%/฿, floor 6,500.00 / ปกติ=7,500.00 @50.00-50.99, step 1.50%/฿</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250฿)</t>
+          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500.00฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250.00฿)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-05-08 18:39
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -26,19 +26,19 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$70</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$106</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Hints_DoubleOrigin'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 18:26</t>
+          <t>2026-05-08 18:39</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>735782.46</v>
+        <v>720918.4</v>
       </c>
     </row>
     <row r="14">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>147751</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="21">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>912806</v>
+        <v>890510</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3305,74 +3305,8 @@
         <v>9750</v>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B76" s="5" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F76" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G76" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H76" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I76" s="6" t="n">
-        <v>11148.03</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F77" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G77" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H77" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I77" s="7" t="n">
-        <v>11148.03</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I77"/>
+  <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3383,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4934,21 +4868,21 @@
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
-        <v>46143</v>
+        <v>46133</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-6802</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>downtime_origin_day</t>
+          <t>midnight_full</t>
         </is>
       </c>
       <c r="E37" s="2" t="n">
@@ -4956,31 +4890,39 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (20.96h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
+          <t>2026-04-21 16:38:59</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-22 13:36:47</t>
+        </is>
+      </c>
       <c r="K37" s="7" t="n">
-        <v>7432.03</v>
+        <v>6645.86</v>
       </c>
       <c r="L37" s="7" t="n">
-        <v>3716</v>
+        <v>6645</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>46143</v>
+        <v>46133</v>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-8681</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -4990,7 +4932,7 @@
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>downtime_origin_day</t>
+          <t>midnight_full</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
@@ -4998,22 +4940,30 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (21.30h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+        </is>
+      </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="J38" s="5" t="inlineStr"/>
+          <t>2026-04-21 13:37:02</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:55:11</t>
+        </is>
+      </c>
       <c r="K38" s="6" t="n">
-        <v>7432.03</v>
+        <v>6645.86</v>
       </c>
       <c r="L38" s="6" t="n">
-        <v>3716</v>
+        <v>6645</v>
       </c>
     </row>
     <row r="39">
@@ -5022,7 +4972,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>71-6802</t>
+          <t>71-9629</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -5046,17 +4996,17 @@
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (20.96h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
+          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (18.79h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>2026-04-21 16:38:59</t>
+          <t>2026-04-21 09:15:51</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 13:36:47</t>
+          <t>2026-04-22 04:03:28</t>
         </is>
       </c>
       <c r="K39" s="7" t="n">
@@ -5066,108 +5016,8 @@
         <v>6645</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>71-8681</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>midnight_full</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr">
-        <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (21.30h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-21 13:37:02</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-22 10:55:11</t>
-        </is>
-      </c>
-      <c r="K40" s="6" t="n">
-        <v>6645.86</v>
-      </c>
-      <c r="L40" s="6" t="n">
-        <v>6645</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="9" t="n">
-        <v>46133</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>71-9629</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>midnight_full</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr"/>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>รอปลายทางข้ามคืน Dest_In→Dest_Out (18.79h); เต็ม 1 เที่ยว (เรทวัน Dest_In)</t>
-        </is>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-21 09:15:51</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-22 04:03:28</t>
-        </is>
-      </c>
-      <c r="K41" s="7" t="n">
-        <v>6645.86</v>
-      </c>
-      <c r="L41" s="7" t="n">
-        <v>6645</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:L39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5609,7 +5459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5667,8 +5517,50 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>71-5042</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>7432.03</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>No matched trip on this trip_date; OAT rule: charge 1 full trip (review before adding to grand total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>72-1217</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>46143</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>7432.03</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>No matched trip on this trip_date; OAT rule: charge 1 full trip (review before adding to grand total)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5777,7 +5669,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>735782.46</v>
+        <v>720918.4</v>
       </c>
     </row>
     <row r="3">
@@ -5837,7 +5729,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>147751</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="7">
@@ -5867,7 +5759,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>912806</v>
+        <v>890510</v>
       </c>
     </row>
   </sheetData>
@@ -5882,7 +5774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6116,19 +6008,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:C20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6139,7 +6020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8752,84 +8633,8 @@
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F69" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G69" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H69" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I69" s="7" t="n">
-        <v>11148.03</v>
-      </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B70" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E70" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="F70" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="G70" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="H70" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="6" t="n">
-        <v>11148.03</v>
-      </c>
-      <c r="J70" s="5" t="inlineStr">
-        <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J70"/>
+  <autoFilter ref="A1:J68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8840,7 +8645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z106"/>
+  <dimension ref="A1:Z104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18103,184 +17908,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
-        </is>
-      </c>
-      <c r="G105" s="2" t="inlineStr">
-        <is>
-          <t>13.8</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr">
-        <is>
-          <t>14.9</t>
-        </is>
-      </c>
-      <c r="I105" s="11" t="n">
-        <v>46143.26266203704</v>
-      </c>
-      <c r="J105" s="11" t="n">
-        <v>46143.48762731482</v>
-      </c>
-      <c r="K105" s="2" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="L105" s="11" t="n">
-        <v>46143.56759259259</v>
-      </c>
-      <c r="M105" s="11" t="n">
-        <v>46143.6196875</v>
-      </c>
-      <c r="N105" s="2" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="O105" s="2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="P105" s="2" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="Q105" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R105" s="2" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="S105" s="2" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="T105" s="2" t="n"/>
-      <c r="U105" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V105" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="W105" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="X105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z105" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="C106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D106" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="E106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="F106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
-        </is>
-      </c>
-      <c r="G106" s="5" t="inlineStr">
-        <is>
-          <t>7.14</t>
-        </is>
-      </c>
-      <c r="H106" s="5" t="inlineStr">
-        <is>
-          <t>7.14</t>
-        </is>
-      </c>
-      <c r="I106" s="10" t="n">
-        <v>46143.82527777777</v>
-      </c>
-      <c r="J106" s="10" t="n">
-        <v>46143.89219907407</v>
-      </c>
-      <c r="K106" s="5" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="L106" s="10" t="n">
-        <v>46143.96318287037</v>
-      </c>
-      <c r="M106" s="10" t="n">
-        <v>46143.97673611111</v>
-      </c>
-      <c r="N106" s="5" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="O106" s="5" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="P106" s="5" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="Q106" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R106" s="5" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="S106" s="5" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="T106" s="5" t="n"/>
-      <c r="U106" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V106" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="W106" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="X106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z106" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Z106"/>
+  <autoFilter ref="A1:Z104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18291,7 +17920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -20915,58 +20544,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C105" s="7" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="D105" s="7" t="n">
-        <v>3716</v>
-      </c>
-      <c r="E105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F105" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" s="7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="8" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B106" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C106" s="6" t="n">
-        <v>7432.03</v>
-      </c>
-      <c r="D106" s="6" t="n">
-        <v>3716</v>
-      </c>
-      <c r="E106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F106" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G106"/>
+  <autoFilter ref="A1:G104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21524,7 +21103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -22136,37 +21715,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>46143</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22177,7 +21727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M73"/>
+  <dimension ref="A1:M71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -25552,102 +25102,8 @@
         <v>15.4</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>71-5042</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="E72" s="5" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G72" s="5" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="H72" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I72" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J72" s="5" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="K72" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="L72" s="5" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="M72" s="5" t="n">
-        <v>15.43</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="F73" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I73" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J73" s="2" t="n">
-        <v>1.61</v>
-      </c>
-      <c r="K73" s="2" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="L73" s="2" t="n">
-        <v>3.63</v>
-      </c>
-      <c r="M73" s="2" t="n">
-        <v>20.37</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:M73"/>
+  <autoFilter ref="A1:M71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Oatside: remove manual_extra_trips 72-1217 apr-22 (7,500 baht) — not in GPS
Total corrected from 890,510 → 883,010 to match Book3.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -25,7 +25,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hints_DoubleOrigin" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$104</definedName>
@@ -35,7 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$4</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08 18:39</t>
+          <t>2026-05-09 00:22</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>720918.4</v>
+        <v>713418.4</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>890510</v>
+        <v>883010</v>
       </c>
     </row>
   </sheetData>
@@ -2825,13 +2825,13 @@
         </is>
       </c>
       <c r="D61" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E61" s="7" t="n">
         <v>6546.17</v>
       </c>
       <c r="F61" s="7" t="n">
-        <v>14046</v>
+        <v>6546.17</v>
       </c>
       <c r="G61" s="7" t="n">
         <v>3273</v>
@@ -2840,7 +2840,7 @@
         <v>0</v>
       </c>
       <c r="I61" s="7" t="n">
-        <v>17319</v>
+        <v>9819</v>
       </c>
     </row>
     <row r="62">
@@ -5028,13 +5028,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="43" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5059,26 +5059,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>46134</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>7500</v>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5632,7 +5614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5669,101 +5651,86 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>720918.4</v>
+        <v>713418.4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>R</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ในนั้น: เที่ยวเพิ่ม (manual_extra_trips ไม่มีใน GPS)</t>
+          <t>ค่าขนส่งขากลับ (manual_return_trips — ไม่เพิ่มจำนวน matched)</t>
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>7500</v>
+        <v>3273.09</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>ค่าขนส่งขากลับ (manual_return_trips — ไม่เพิ่มจำนวน matched)</t>
+          <t>ค่าชดเชยเที่ยวขาด (min 2/คัน/วัน) — ไม่เก็บเงิน (ใช้ชาร์จ 50% วันละ 1 เที่ยวแทน)</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>3273.09</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ค่าชดเชยเที่ยวขาด (min 2/คัน/วัน) — ไม่เก็บเงิน (ใช้ชาร์จ 50% วันละ 1 เที่ยวแทน)</t>
+          <t>ชาร์จ 50% วันที่วิ่งได้ 1 เที่ยว (หลัง override)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0</v>
+        <v>140319</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>ชาร์จ 50% วันที่วิ่งได้ 1 เที่ยว (หลัง override)</t>
+          <t>No-work recovery outbound 50pct (first matched trip that Dest_In day on recovery dates)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>140319</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>No-work recovery outbound 50pct (first matched trip that Dest_In day on recovery dates)</t>
+          <t>Grand (A+C+D+R)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>26000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Grand (A+C+D+R)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>890510</v>
+        <v>883010</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C8"/>
+  <autoFilter ref="A1:C7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5947,7 +5914,7 @@
         <v>46134</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>4</v>
@@ -8192,13 +8159,13 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" s="7" t="n">
         <v>6546.17</v>
       </c>
       <c r="F57" s="7" t="n">
-        <v>14046</v>
+        <v>6546.17</v>
       </c>
       <c r="G57" s="7" t="n">
         <v>3273</v>
@@ -8207,11 +8174,11 @@
         <v>3273</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>20592</v>
+        <v>13092</v>
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | เที่ยวเพิ่ม (ไม่มีใน GPS): P&amp;G → Oatside (เที่ยวเพิ่ม — ไม่มีใน GPS) (+7,500.00฿) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,273.09฿)</t>
+          <t>เก็บ 50% อัตโนมัติ (วันงาน 1 เที่ยว) | ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,273.09฿)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oatside Pages: deploy report with BH +29,440 + +0฿ fix to oatside-pg-2026
Sync fresh build (Oatside/TransportRateCalculator/reports/oatside-apr2026) into the
GitHub Pages folder reports/oatside-pg-2026 so the public link shows the backhaul
revenue + the manual_return render fix. Targeted copy (overwrite index/trips/exports/
plates) — preserves discrepancy_check.html & manual_check.html, which the full-replace
deploy_oatside_report.ps1 would have deleted.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -36,7 +36,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$125</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Phantom_Trip_Candidates'!$A$1:$E$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Hints_DoubleOrigin'!$A$1:$D$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-05 22:49</t>
+          <t>2026-06-08 18:49</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>3250</v>
+        <v>32690</v>
       </c>
     </row>
     <row r="16">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1469970</v>
+        <v>1499410</v>
       </c>
     </row>
   </sheetData>
@@ -923,10 +923,10 @@
         <v>3632</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="4">
@@ -1946,10 +1946,10 @@
         <v>3584</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
     </row>
     <row r="35">
@@ -2045,10 +2045,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14336</v>
+        <v>17920</v>
       </c>
     </row>
     <row r="38">
@@ -3068,10 +3068,10 @@
         <v>3728</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="69">
@@ -3101,10 +3101,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="70">
@@ -3167,10 +3167,10 @@
         <v>3728</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="72">
@@ -3233,10 +3233,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="74">
@@ -3497,10 +3497,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
     </row>
     <row r="82">
@@ -8587,13 +8587,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="41" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8636,8 +8636,152 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="9" t="n">
+        <v>46143</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>71-5042</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3632</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>ตีเปล่าไป P&amp;G 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>46152</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>3584</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>71-8002</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>71-8001</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับเพิ่ม 50% (base คิด ตีเปล่า+BH#1 = 1 เที่ยวแล้ว)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>71-8001</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>3728</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>BH ขากลับ P&amp;G&gt;บ้านบึง 50%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8853,7 +8997,7 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>3250</v>
+        <v>32690</v>
       </c>
     </row>
     <row r="4">
@@ -8913,7 +9057,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1469970</v>
+        <v>1499410</v>
       </c>
     </row>
   </sheetData>
@@ -9400,14 +9544,14 @@
         <v>0</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>0</v>
+        <v>3250</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>0</v>
+        <v>3250</v>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+0.00฿)</t>
+          <t>ขากลับ (manual): ค่าขนส่งงานขากลับ 50% ของราคาเที่ยวหลัก (+3,250.00฿)</t>
         </is>
       </c>
     </row>
@@ -9438,14 +9582,14 @@
         <v>3632</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): ตีเปล่าไป P&amp;G 50% (+3,632.00฿)</t>
         </is>
       </c>
     </row>
@@ -10616,14 +10760,14 @@
         <v>3584</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>10752</v>
+        <v>14336</v>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,584.00฿)</t>
         </is>
       </c>
     </row>
@@ -10730,14 +10874,14 @@
         <v>0</v>
       </c>
       <c r="H37" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
       <c r="I37" s="7" t="n">
-        <v>14336</v>
+        <v>17920</v>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,584.00฿)</t>
         </is>
       </c>
     </row>
@@ -11908,14 +12052,14 @@
         <v>3728</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I68" s="6" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
       <c r="J68" s="5" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับเพิ่ม 50% (base คิด ตีเปล่า+BH#1 = 1 เที่ยวแล้ว) (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -11946,14 +12090,14 @@
         <v>0</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12022,14 +12166,14 @@
         <v>3728</v>
       </c>
       <c r="H71" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>11184</v>
+        <v>14912</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12098,14 +12242,14 @@
         <v>0</v>
       </c>
       <c r="H73" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I73" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -12402,14 +12546,14 @@
         <v>0</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
       <c r="I81" s="7" t="n">
-        <v>14912</v>
+        <v>18640</v>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว)</t>
+          <t>ไม่เก็บเพิ่ม (จบ 2 เที่ยว) | ขากลับ (manual): BH ขากลับ P&amp;G&gt;บ้านบึง 50% (+3,728.00฿)</t>
         </is>
       </c>
     </row>
@@ -14345,7 +14489,7 @@
         <v>0</v>
       </c>
       <c r="Z2" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="3">
@@ -17249,7 +17393,7 @@
         <v>0</v>
       </c>
       <c r="Z35" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="36">
@@ -17601,7 +17745,7 @@
         <v>0</v>
       </c>
       <c r="Z39" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="40">
@@ -21477,7 +21621,7 @@
         <v>0</v>
       </c>
       <c r="Z83" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="84">
@@ -21565,7 +21709,7 @@
         <v>0</v>
       </c>
       <c r="Z84" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="85">
@@ -21917,7 +22061,7 @@
         <v>0</v>
       </c>
       <c r="Z88" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="89">
@@ -22093,7 +22237,7 @@
         <v>0</v>
       </c>
       <c r="Z90" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="91">
@@ -22885,7 +23029,7 @@
         <v>0</v>
       </c>
       <c r="Z99" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="100">
@@ -27911,7 +28055,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="3">
@@ -28736,7 +28880,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="36">
@@ -28836,7 +28980,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>0</v>
+        <v>3584</v>
       </c>
     </row>
     <row r="40">
@@ -29936,7 +30080,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="84">
@@ -29961,7 +30105,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="85">
@@ -30061,7 +30205,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="89">
@@ -30111,7 +30255,7 @@
         <v>0</v>
       </c>
       <c r="G90" s="6" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="91">
@@ -30336,7 +30480,7 @@
         <v>0</v>
       </c>
       <c r="G99" s="7" t="n">
-        <v>0</v>
+        <v>3728</v>
       </c>
     </row>
     <row r="100">

</xml_diff>

<commit_message>
Oatside May 2026: remove phantom trip 71-8009 28/05 (truck did not run) - grand 1,485,120
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -28,13 +28,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Customer_Summary'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Customer_Trips_Per_Day'!$A$1:$C$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Audit_Log'!$A$1:$J$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$154</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Trip_Detail'!$A$1:$Z$153</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Trips_Pricing_All'!$A$1:$G$153</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$124</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$123</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-06-09 15:05</t>
+          <t>2026-06-10 13:46</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1121952</v>
+        <v>1114592</v>
       </c>
     </row>
     <row r="14">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>337312</v>
+        <v>333632</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1496160</v>
+        <v>1485120</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I124"/>
+  <dimension ref="A1:I123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4400,12 +4400,12 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
@@ -4429,35 +4429,35 @@
     </row>
     <row r="110">
       <c r="A110" s="8" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E110" s="6" t="n">
         <v>7360</v>
       </c>
       <c r="F110" s="6" t="n">
-        <v>7360</v>
+        <v>14720</v>
       </c>
       <c r="G110" s="6" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H110" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I110" s="6" t="n">
-        <v>11040</v>
+        <v>14720</v>
       </c>
     </row>
     <row r="111">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -4565,64 +4565,64 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E114" s="6" t="n">
         <v>7360</v>
       </c>
       <c r="F114" s="6" t="n">
-        <v>14720</v>
+        <v>7360</v>
       </c>
       <c r="G114" s="6" t="n">
-        <v>0</v>
+        <v>3680</v>
       </c>
       <c r="H114" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I114" s="6" t="n">
-        <v>14720</v>
+        <v>11040</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
         <v>1</v>
       </c>
       <c r="E115" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="F115" s="7" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="G115" s="7" t="n">
-        <v>3680</v>
+        <v>3632</v>
       </c>
       <c r="H115" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I115" s="7" t="n">
-        <v>11040</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="116">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
@@ -4640,22 +4640,22 @@
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E116" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="F116" s="6" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G116" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H116" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I116" s="6" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="117">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -4673,22 +4673,22 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E117" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F117" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G117" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H117" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I117" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="118">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -4730,45 +4730,45 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E119" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F119" s="7" t="n">
-        <v>7264</v>
+        <v>14528</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I119" s="7" t="n">
-        <v>10896</v>
+        <v>14528</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -4805,22 +4805,22 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="F121" s="7" t="n">
-        <v>14528</v>
+        <v>7264</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>14528</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="122">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -4862,12 +4862,12 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
@@ -4889,41 +4889,8 @@
         <v>10896</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B124" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="F124" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="G124" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="H124" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I124" s="6" t="n">
-        <v>10896</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I124"/>
+  <autoFilter ref="A1:I123"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4934,7 +4901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8127,12 +8094,12 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
@@ -8165,7 +8132,7 @@
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -8194,7 +8161,7 @@
       <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
@@ -8207,16 +8174,16 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
@@ -8236,15 +8203,15 @@
       <c r="H78" s="5" t="inlineStr"/>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr"/>
       <c r="K78" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="L78" s="6" t="n">
-        <v>3680</v>
+        <v>3632</v>
       </c>
     </row>
     <row r="79">
@@ -8253,7 +8220,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8295,7 +8262,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -8333,11 +8300,11 @@
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -8362,7 +8329,7 @@
       <c r="H81" s="2" t="inlineStr"/>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
@@ -8379,7 +8346,7 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -8421,12 +8388,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -8457,50 +8424,8 @@
         <v>3632</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B84" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>one_trip_billed_day</t>
-        </is>
-      </c>
-      <c r="E84" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F84" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G84" s="5" t="inlineStr"/>
-      <c r="H84" s="5" t="inlineStr"/>
-      <c r="I84" s="5" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="J84" s="5" t="inlineStr"/>
-      <c r="K84" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="L84" s="6" t="n">
-        <v>3632</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L84"/>
+  <autoFilter ref="A1:L83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8967,7 +8892,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1121952</v>
+        <v>1114592</v>
       </c>
     </row>
     <row r="3">
@@ -9027,7 +8952,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>337312</v>
+        <v>333632</v>
       </c>
     </row>
     <row r="7">
@@ -9057,7 +8982,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1496160</v>
+        <v>1485120</v>
       </c>
     </row>
   </sheetData>
@@ -9399,10 +9324,10 @@
         <v>46170</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30">
@@ -13598,26 +13523,26 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E109" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="F109" s="7" t="n">
-        <v>7360</v>
+        <v>0</v>
       </c>
       <c r="G109" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="H109" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I109" s="7" t="n">
-        <v>11040</v>
+        <v>0</v>
       </c>
       <c r="J109" s="2" t="inlineStr">
         <is>
-          <t>เก็บ 50% อัตโนมัติ (จบ 1 เที่ยว)</t>
+          <t>ไม่เก็บ [override: exclude_50] — รถไม่ได้วิ่งจริง — ตัดเที่ยวเดียวของวันออกจาก base แล้ว เหลือ 0 เที่ยว แต่ GPS เห็นรถที่โรงงาน → กัน no_finish 100% ลั่น (คู่กับ remove_matched_trips ใน oatside_config.json)</t>
         </is>
       </c>
     </row>
@@ -14203,7 +14128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z154"/>
+  <dimension ref="A1:Z153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25992,7 +25917,7 @@
     </row>
     <row r="134">
       <c r="A134" s="8" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B134" s="8" t="n">
         <v>46170</v>
@@ -26002,67 +25927,63 @@
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G134" s="5" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="H134" s="5" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>2.37</t>
         </is>
       </c>
       <c r="I134" s="10" t="n">
-        <v>46170.11607638889</v>
+        <v>46170.58722222222</v>
       </c>
       <c r="J134" s="10" t="n">
-        <v>46170.26921296296</v>
+        <v>46170.89265046296</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>3.68</v>
+        <v>7.33</v>
       </c>
       <c r="L134" s="10" t="n">
-        <v>46170.83622685185</v>
+        <v>46170.96063657408</v>
       </c>
       <c r="M134" s="10" t="n">
-        <v>46170.9013425926</v>
+        <v>46171.30994212963</v>
       </c>
       <c r="N134" s="5" t="n">
-        <v>13.61</v>
+        <v>1.63</v>
       </c>
       <c r="O134" s="5" t="n">
-        <v>1.56</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="P134" s="5" t="n">
-        <v>1.56</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="Q134" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R134" s="5" t="n">
-        <v>18.85</v>
+        <v>17.35</v>
       </c>
       <c r="S134" s="5" t="n">
-        <v>18.85</v>
-      </c>
-      <c r="T134" s="5" t="inlineStr">
-        <is>
-          <t>ABNORMAL</t>
-        </is>
-      </c>
+        <v>17.35</v>
+      </c>
+      <c r="T134" s="5" t="n"/>
       <c r="U134" s="5" t="n">
         <v>1</v>
       </c>
@@ -26087,68 +26008,68 @@
         <v>46171</v>
       </c>
       <c r="B135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="C135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>2.37</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="I135" s="11" t="n">
-        <v>46170.58722222222</v>
+        <v>46171.16535879629</v>
       </c>
       <c r="J135" s="11" t="n">
-        <v>46170.89265046296</v>
+        <v>46171.27927083334</v>
       </c>
       <c r="K135" s="2" t="n">
-        <v>7.33</v>
+        <v>2.73</v>
       </c>
       <c r="L135" s="11" t="n">
-        <v>46170.96063657408</v>
+        <v>46171.37247685185</v>
       </c>
       <c r="M135" s="11" t="n">
-        <v>46171.30994212963</v>
+        <v>46171.61934027778</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>1.63</v>
+        <v>2.24</v>
       </c>
       <c r="O135" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>5.92</v>
       </c>
       <c r="P135" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>5.92</v>
       </c>
       <c r="Q135" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R135" s="2" t="n">
-        <v>17.35</v>
+        <v>10.9</v>
       </c>
       <c r="S135" s="2" t="n">
-        <v>17.35</v>
+        <v>10.9</v>
       </c>
       <c r="T135" s="2" t="n"/>
       <c r="U135" s="2" t="n">
@@ -26158,7 +26079,7 @@
         <v>7360</v>
       </c>
       <c r="W135" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="X135" s="7" t="n">
         <v>0</v>
@@ -26197,46 +26118,46 @@
       </c>
       <c r="G136" s="5" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="H136" s="5" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="I136" s="10" t="n">
-        <v>46171.16535879629</v>
+        <v>46171.78201388889</v>
       </c>
       <c r="J136" s="10" t="n">
-        <v>46171.27927083334</v>
+        <v>46171.89481481481</v>
       </c>
       <c r="K136" s="5" t="n">
-        <v>2.73</v>
+        <v>2.71</v>
       </c>
       <c r="L136" s="10" t="n">
-        <v>46171.37247685185</v>
+        <v>46171.96677083334</v>
       </c>
       <c r="M136" s="10" t="n">
-        <v>46171.61934027778</v>
+        <v>46172.09275462963</v>
       </c>
       <c r="N136" s="5" t="n">
-        <v>2.24</v>
+        <v>1.73</v>
       </c>
       <c r="O136" s="5" t="n">
-        <v>5.92</v>
+        <v>3.02</v>
       </c>
       <c r="P136" s="5" t="n">
-        <v>5.92</v>
+        <v>3.02</v>
       </c>
       <c r="Q136" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R136" s="5" t="n">
-        <v>10.9</v>
+        <v>7.46</v>
       </c>
       <c r="S136" s="5" t="n">
-        <v>10.9</v>
+        <v>7.46</v>
       </c>
       <c r="T136" s="5" t="n"/>
       <c r="U136" s="5" t="n">
@@ -26275,56 +26196,56 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>7.25</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>8.28</t>
         </is>
       </c>
       <c r="I137" s="11" t="n">
-        <v>46171.78201388889</v>
+        <v>46171.33181712963</v>
       </c>
       <c r="J137" s="11" t="n">
-        <v>46171.89481481481</v>
+        <v>46171.60032407408</v>
       </c>
       <c r="K137" s="2" t="n">
-        <v>2.71</v>
+        <v>6.44</v>
       </c>
       <c r="L137" s="11" t="n">
-        <v>46171.96677083334</v>
+        <v>46171.67759259259</v>
       </c>
       <c r="M137" s="11" t="n">
-        <v>46172.09275462963</v>
+        <v>46171.70689814815</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>1.73</v>
+        <v>1.85</v>
       </c>
       <c r="O137" s="2" t="n">
-        <v>3.02</v>
+        <v>0.7</v>
       </c>
       <c r="P137" s="2" t="n">
-        <v>3.02</v>
+        <v>0.7</v>
       </c>
       <c r="Q137" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R137" s="2" t="n">
-        <v>7.46</v>
+        <v>9</v>
       </c>
       <c r="S137" s="2" t="n">
-        <v>7.46</v>
+        <v>9</v>
       </c>
       <c r="T137" s="2" t="n"/>
       <c r="U137" s="2" t="n">
@@ -26351,7 +26272,7 @@
         <v>46171</v>
       </c>
       <c r="B138" s="8" t="n">
-        <v>46171</v>
+        <v>46170</v>
       </c>
       <c r="C138" s="8" t="n">
         <v>46171</v>
@@ -26363,56 +26284,56 @@
       </c>
       <c r="E138" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8003 โกสินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G138" s="5" t="inlineStr">
         <is>
-          <t>7.25</t>
+          <t>10.4</t>
         </is>
       </c>
       <c r="H138" s="5" t="inlineStr">
         <is>
-          <t>8.28</t>
+          <t>11.4</t>
         </is>
       </c>
       <c r="I138" s="10" t="n">
-        <v>46171.33181712963</v>
+        <v>46170.99238425926</v>
       </c>
       <c r="J138" s="10" t="n">
-        <v>46171.60032407408</v>
+        <v>46171.28165509259</v>
       </c>
       <c r="K138" s="5" t="n">
-        <v>6.44</v>
+        <v>6.94</v>
       </c>
       <c r="L138" s="10" t="n">
-        <v>46171.67759259259</v>
+        <v>46171.3696875</v>
       </c>
       <c r="M138" s="10" t="n">
-        <v>46171.70689814815</v>
+        <v>46171.59075231481</v>
       </c>
       <c r="N138" s="5" t="n">
-        <v>1.85</v>
+        <v>2.11</v>
       </c>
       <c r="O138" s="5" t="n">
-        <v>0.7</v>
+        <v>5.31</v>
       </c>
       <c r="P138" s="5" t="n">
-        <v>0.7</v>
+        <v>5.31</v>
       </c>
       <c r="Q138" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R138" s="5" t="n">
-        <v>9</v>
+        <v>14.36</v>
       </c>
       <c r="S138" s="5" t="n">
-        <v>9</v>
+        <v>14.36</v>
       </c>
       <c r="T138" s="5" t="n"/>
       <c r="U138" s="5" t="n">
@@ -26439,7 +26360,7 @@
         <v>46171</v>
       </c>
       <c r="B139" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="C139" s="9" t="n">
         <v>46171</v>
@@ -26461,46 +26382,46 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>11.4</t>
+          <t>11.5</t>
         </is>
       </c>
       <c r="I139" s="11" t="n">
-        <v>46170.99238425926</v>
+        <v>46171.66229166667</v>
       </c>
       <c r="J139" s="11" t="n">
-        <v>46171.28165509259</v>
+        <v>46171.72710648148</v>
       </c>
       <c r="K139" s="2" t="n">
-        <v>6.94</v>
+        <v>1.56</v>
       </c>
       <c r="L139" s="11" t="n">
-        <v>46171.3696875</v>
+        <v>46171.82959490741</v>
       </c>
       <c r="M139" s="11" t="n">
-        <v>46171.59075231481</v>
+        <v>46171.94225694444</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>2.11</v>
+        <v>2.46</v>
       </c>
       <c r="O139" s="2" t="n">
-        <v>5.31</v>
+        <v>2.7</v>
       </c>
       <c r="P139" s="2" t="n">
-        <v>5.31</v>
+        <v>2.7</v>
       </c>
       <c r="Q139" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R139" s="2" t="n">
-        <v>14.36</v>
+        <v>6.72</v>
       </c>
       <c r="S139" s="2" t="n">
-        <v>14.36</v>
+        <v>6.72</v>
       </c>
       <c r="T139" s="2" t="n"/>
       <c r="U139" s="2" t="n">
@@ -26539,56 +26460,56 @@
       </c>
       <c r="E140" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
-          <t>71-8003 โกสินทร์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G140" s="5" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>5.25</t>
         </is>
       </c>
       <c r="H140" s="5" t="inlineStr">
         <is>
-          <t>11.5</t>
+          <t>5.25</t>
         </is>
       </c>
       <c r="I140" s="10" t="n">
-        <v>46171.66229166667</v>
+        <v>46171.00243055556</v>
       </c>
       <c r="J140" s="10" t="n">
-        <v>46171.72710648148</v>
+        <v>46171.46831018518</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>1.56</v>
+        <v>11.18</v>
       </c>
       <c r="L140" s="10" t="n">
-        <v>46171.82959490741</v>
+        <v>46171.54582175926</v>
       </c>
       <c r="M140" s="10" t="n">
-        <v>46171.94225694444</v>
+        <v>46171.60834490741</v>
       </c>
       <c r="N140" s="5" t="n">
-        <v>2.46</v>
+        <v>1.86</v>
       </c>
       <c r="O140" s="5" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="P140" s="5" t="n">
-        <v>2.7</v>
+        <v>1.5</v>
       </c>
       <c r="Q140" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R140" s="5" t="n">
-        <v>6.72</v>
+        <v>14.54</v>
       </c>
       <c r="S140" s="5" t="n">
-        <v>6.72</v>
+        <v>14.54</v>
       </c>
       <c r="T140" s="5" t="n"/>
       <c r="U140" s="5" t="n">
@@ -26637,46 +26558,46 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>5.26</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>5.26</t>
         </is>
       </c>
       <c r="I141" s="11" t="n">
-        <v>46171.00243055556</v>
+        <v>46171.67638888889</v>
       </c>
       <c r="J141" s="11" t="n">
-        <v>46171.46831018518</v>
+        <v>46171.7416087963</v>
       </c>
       <c r="K141" s="2" t="n">
-        <v>11.18</v>
+        <v>1.57</v>
       </c>
       <c r="L141" s="11" t="n">
-        <v>46171.54582175926</v>
+        <v>46171.82641203704</v>
       </c>
       <c r="M141" s="11" t="n">
-        <v>46171.60834490741</v>
+        <v>46171.875625</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>1.86</v>
+        <v>2.04</v>
       </c>
       <c r="O141" s="2" t="n">
-        <v>1.5</v>
+        <v>1.18</v>
       </c>
       <c r="P141" s="2" t="n">
-        <v>1.5</v>
+        <v>1.18</v>
       </c>
       <c r="Q141" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R141" s="2" t="n">
-        <v>14.54</v>
+        <v>4.78</v>
       </c>
       <c r="S141" s="2" t="n">
-        <v>14.54</v>
+        <v>4.78</v>
       </c>
       <c r="T141" s="2" t="n"/>
       <c r="U141" s="2" t="n">
@@ -26700,7 +26621,7 @@
     </row>
     <row r="142">
       <c r="A142" s="8" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B142" s="8" t="n">
         <v>46171</v>
@@ -26710,68 +26631,68 @@
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G142" s="5" t="inlineStr">
         <is>
-          <t>5.26</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="H142" s="5" t="inlineStr">
         <is>
-          <t>5.26</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="I142" s="10" t="n">
-        <v>46171.67638888889</v>
+        <v>46171.72065972222</v>
       </c>
       <c r="J142" s="10" t="n">
-        <v>46171.7416087963</v>
+        <v>46171.87474537037</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>1.57</v>
+        <v>3.7</v>
       </c>
       <c r="L142" s="10" t="n">
-        <v>46171.82641203704</v>
+        <v>46171.94614583333</v>
       </c>
       <c r="M142" s="10" t="n">
-        <v>46171.875625</v>
+        <v>46172.63309027778</v>
       </c>
       <c r="N142" s="5" t="n">
-        <v>2.04</v>
+        <v>1.71</v>
       </c>
       <c r="O142" s="5" t="n">
-        <v>1.18</v>
+        <v>16.49</v>
       </c>
       <c r="P142" s="5" t="n">
-        <v>1.18</v>
+        <v>16.49</v>
       </c>
       <c r="Q142" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R142" s="5" t="n">
-        <v>4.78</v>
+        <v>21.9</v>
       </c>
       <c r="S142" s="5" t="n">
-        <v>4.78</v>
+        <v>21.9</v>
       </c>
       <c r="T142" s="5" t="n"/>
       <c r="U142" s="5" t="n">
         <v>1</v>
       </c>
       <c r="V142" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="W142" s="6" t="n">
         <v>0</v>
@@ -26791,68 +26712,68 @@
         <v>46172</v>
       </c>
       <c r="B143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="C143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>2.38</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="I143" s="11" t="n">
-        <v>46171.72065972222</v>
+        <v>46172.32059027778</v>
       </c>
       <c r="J143" s="11" t="n">
-        <v>46171.87474537037</v>
+        <v>46172.47302083333</v>
       </c>
       <c r="K143" s="2" t="n">
-        <v>3.7</v>
+        <v>3.66</v>
       </c>
       <c r="L143" s="11" t="n">
-        <v>46171.94614583333</v>
+        <v>46172.56171296296</v>
       </c>
       <c r="M143" s="11" t="n">
-        <v>46172.63309027778</v>
+        <v>46172.81743055556</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>1.71</v>
+        <v>2.13</v>
       </c>
       <c r="O143" s="2" t="n">
-        <v>16.49</v>
+        <v>6.14</v>
       </c>
       <c r="P143" s="2" t="n">
-        <v>16.49</v>
+        <v>6.14</v>
       </c>
       <c r="Q143" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R143" s="2" t="n">
-        <v>21.9</v>
+        <v>11.92</v>
       </c>
       <c r="S143" s="2" t="n">
-        <v>21.9</v>
+        <v>11.92</v>
       </c>
       <c r="T143" s="2" t="n"/>
       <c r="U143" s="2" t="n">
@@ -26862,7 +26783,7 @@
         <v>7264</v>
       </c>
       <c r="W143" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X143" s="7" t="n">
         <v>0</v>
@@ -26879,7 +26800,7 @@
         <v>46172</v>
       </c>
       <c r="B144" s="8" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="C144" s="8" t="n">
         <v>46172</v>
@@ -26891,58 +26812,62 @@
       </c>
       <c r="E144" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F144" s="5" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G144" s="5" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>7.26</t>
         </is>
       </c>
       <c r="H144" s="5" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>8.29</t>
         </is>
       </c>
       <c r="I144" s="10" t="n">
-        <v>46172.32059027778</v>
+        <v>46171.82071759259</v>
       </c>
       <c r="J144" s="10" t="n">
-        <v>46172.47302083333</v>
+        <v>46171.92391203704</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>3.66</v>
+        <v>2.48</v>
       </c>
       <c r="L144" s="10" t="n">
-        <v>46172.56171296296</v>
+        <v>46172.29966435185</v>
       </c>
       <c r="M144" s="10" t="n">
-        <v>46172.81743055556</v>
+        <v>46172.37111111111</v>
       </c>
       <c r="N144" s="5" t="n">
-        <v>2.13</v>
+        <v>9.02</v>
       </c>
       <c r="O144" s="5" t="n">
-        <v>6.14</v>
+        <v>1.71</v>
       </c>
       <c r="P144" s="5" t="n">
-        <v>6.14</v>
+        <v>1.71</v>
       </c>
       <c r="Q144" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R144" s="5" t="n">
-        <v>11.92</v>
+        <v>13.21</v>
       </c>
       <c r="S144" s="5" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="T144" s="5" t="n"/>
+        <v>13.21</v>
+      </c>
+      <c r="T144" s="5" t="inlineStr">
+        <is>
+          <t>ABNORMAL</t>
+        </is>
+      </c>
       <c r="U144" s="5" t="n">
         <v>1</v>
       </c>
@@ -26950,7 +26875,7 @@
         <v>7264</v>
       </c>
       <c r="W144" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X144" s="6" t="n">
         <v>0</v>
@@ -26967,7 +26892,7 @@
         <v>46172</v>
       </c>
       <c r="B145" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="C145" s="9" t="n">
         <v>46172</v>
@@ -26989,52 +26914,48 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>7.26</t>
+          <t>7.27</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>8.29</t>
+          <t>8.30</t>
         </is>
       </c>
       <c r="I145" s="11" t="n">
-        <v>46171.82071759259</v>
+        <v>46172.43083333333</v>
       </c>
       <c r="J145" s="11" t="n">
-        <v>46171.92391203704</v>
+        <v>46172.52552083333</v>
       </c>
       <c r="K145" s="2" t="n">
-        <v>2.48</v>
+        <v>2.27</v>
       </c>
       <c r="L145" s="11" t="n">
-        <v>46172.29966435185</v>
+        <v>46172.61280092593</v>
       </c>
       <c r="M145" s="11" t="n">
-        <v>46172.37111111111</v>
+        <v>46172.86035879629</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>9.02</v>
+        <v>2.09</v>
       </c>
       <c r="O145" s="2" t="n">
-        <v>1.71</v>
+        <v>5.94</v>
       </c>
       <c r="P145" s="2" t="n">
-        <v>1.71</v>
+        <v>5.94</v>
       </c>
       <c r="Q145" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R145" s="2" t="n">
-        <v>13.21</v>
+        <v>10.31</v>
       </c>
       <c r="S145" s="2" t="n">
-        <v>13.21</v>
-      </c>
-      <c r="T145" s="2" t="inlineStr">
-        <is>
-          <t>ABNORMAL</t>
-        </is>
-      </c>
+        <v>10.31</v>
+      </c>
+      <c r="T145" s="2" t="n"/>
       <c r="U145" s="2" t="n">
         <v>1</v>
       </c>
@@ -27071,56 +26992,56 @@
       </c>
       <c r="E146" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="F146" s="5" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8003 โกสินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G146" s="5" t="inlineStr">
         <is>
-          <t>7.27</t>
+          <t>10.6</t>
         </is>
       </c>
       <c r="H146" s="5" t="inlineStr">
         <is>
-          <t>8.30</t>
+          <t>11.6</t>
         </is>
       </c>
       <c r="I146" s="10" t="n">
-        <v>46172.43083333333</v>
+        <v>46172.03034722222</v>
       </c>
       <c r="J146" s="10" t="n">
-        <v>46172.52552083333</v>
+        <v>46172.28571759259</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>2.27</v>
+        <v>6.13</v>
       </c>
       <c r="L146" s="10" t="n">
-        <v>46172.61280092593</v>
+        <v>46172.36446759259</v>
       </c>
       <c r="M146" s="10" t="n">
-        <v>46172.86035879629</v>
+        <v>46172.49165509259</v>
       </c>
       <c r="N146" s="5" t="n">
-        <v>2.09</v>
+        <v>1.89</v>
       </c>
       <c r="O146" s="5" t="n">
-        <v>5.94</v>
+        <v>3.05</v>
       </c>
       <c r="P146" s="5" t="n">
-        <v>5.94</v>
+        <v>3.05</v>
       </c>
       <c r="Q146" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R146" s="5" t="n">
-        <v>10.31</v>
+        <v>11.07</v>
       </c>
       <c r="S146" s="5" t="n">
-        <v>10.31</v>
+        <v>11.07</v>
       </c>
       <c r="T146" s="5" t="n"/>
       <c r="U146" s="5" t="n">
@@ -27130,7 +27051,7 @@
         <v>7264</v>
       </c>
       <c r="W146" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X146" s="6" t="n">
         <v>0</v>
@@ -27147,7 +27068,7 @@
         <v>46172</v>
       </c>
       <c r="B147" s="9" t="n">
-        <v>46172</v>
+        <v>46171</v>
       </c>
       <c r="C147" s="9" t="n">
         <v>46172</v>
@@ -27159,56 +27080,56 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>71-8003 โกสินทร์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>10.6</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="I147" s="11" t="n">
-        <v>46172.03034722222</v>
+        <v>46171.99543981482</v>
       </c>
       <c r="J147" s="11" t="n">
-        <v>46172.28571759259</v>
+        <v>46172.2858449074</v>
       </c>
       <c r="K147" s="2" t="n">
-        <v>6.13</v>
+        <v>6.97</v>
       </c>
       <c r="L147" s="11" t="n">
-        <v>46172.36446759259</v>
+        <v>46172.40947916666</v>
       </c>
       <c r="M147" s="11" t="n">
-        <v>46172.49165509259</v>
+        <v>46172.62247685185</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>1.89</v>
+        <v>2.97</v>
       </c>
       <c r="O147" s="2" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="P147" s="2" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="Q147" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R147" s="2" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="S147" s="2" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="T147" s="2" t="n"/>
       <c r="U147" s="2" t="n">
@@ -27232,13 +27153,13 @@
     </row>
     <row r="148">
       <c r="A148" s="8" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B148" s="8" t="n">
         <v>46172</v>
       </c>
-      <c r="B148" s="8" t="n">
-        <v>46171</v>
-      </c>
       <c r="C148" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
@@ -27247,56 +27168,56 @@
       </c>
       <c r="E148" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="F148" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>71-5042 ณัชพน หัวลาก10W</t>
         </is>
       </c>
       <c r="G148" s="5" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="H148" s="5" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="I148" s="10" t="n">
-        <v>46171.99543981482</v>
+        <v>46172.945</v>
       </c>
       <c r="J148" s="10" t="n">
-        <v>46172.2858449074</v>
+        <v>46173.25171296296</v>
       </c>
       <c r="K148" s="5" t="n">
-        <v>6.97</v>
+        <v>7.36</v>
       </c>
       <c r="L148" s="10" t="n">
-        <v>46172.40947916666</v>
+        <v>46173.33864583333</v>
       </c>
       <c r="M148" s="10" t="n">
-        <v>46172.62247685185</v>
+        <v>46173.38333333333</v>
       </c>
       <c r="N148" s="5" t="n">
-        <v>2.97</v>
+        <v>2.09</v>
       </c>
       <c r="O148" s="5" t="n">
-        <v>5.11</v>
+        <v>1.07</v>
       </c>
       <c r="P148" s="5" t="n">
-        <v>5.11</v>
+        <v>1.07</v>
       </c>
       <c r="Q148" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R148" s="5" t="n">
-        <v>15.05</v>
+        <v>10.52</v>
       </c>
       <c r="S148" s="5" t="n">
-        <v>15.05</v>
+        <v>10.52</v>
       </c>
       <c r="T148" s="5" t="n"/>
       <c r="U148" s="5" t="n">
@@ -27306,7 +27227,7 @@
         <v>7264</v>
       </c>
       <c r="W148" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X148" s="6" t="n">
         <v>0</v>
@@ -27323,7 +27244,7 @@
         <v>46173</v>
       </c>
       <c r="B149" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="C149" s="9" t="n">
         <v>46173</v>
@@ -27345,46 +27266,46 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.9</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="I149" s="11" t="n">
-        <v>46172.945</v>
+        <v>46173.50255787037</v>
       </c>
       <c r="J149" s="11" t="n">
-        <v>46173.25171296296</v>
+        <v>46173.72892361111</v>
       </c>
       <c r="K149" s="2" t="n">
-        <v>7.36</v>
+        <v>5.43</v>
       </c>
       <c r="L149" s="11" t="n">
-        <v>46173.33864583333</v>
+        <v>46173.81170138889</v>
       </c>
       <c r="M149" s="11" t="n">
-        <v>46173.38333333333</v>
+        <v>46173.91047453704</v>
       </c>
       <c r="N149" s="2" t="n">
-        <v>2.09</v>
+        <v>1.99</v>
       </c>
       <c r="O149" s="2" t="n">
-        <v>1.07</v>
+        <v>2.37</v>
       </c>
       <c r="P149" s="2" t="n">
-        <v>1.07</v>
+        <v>2.37</v>
       </c>
       <c r="Q149" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R149" s="2" t="n">
-        <v>10.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="S149" s="2" t="n">
-        <v>10.52</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="T149" s="2" t="n"/>
       <c r="U149" s="2" t="n">
@@ -27411,7 +27332,7 @@
         <v>46173</v>
       </c>
       <c r="B150" s="8" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="C150" s="8" t="n">
         <v>46173</v>
@@ -27423,56 +27344,56 @@
       </c>
       <c r="E150" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="F150" s="5" t="inlineStr">
         <is>
-          <t>71-5042 ณัชพน หัวลาก10W</t>
+          <t>71-8002 สมประสงค์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="H150" s="5" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>8.31</t>
         </is>
       </c>
       <c r="I150" s="10" t="n">
-        <v>46173.50255787037</v>
+        <v>46172.96576388889</v>
       </c>
       <c r="J150" s="10" t="n">
-        <v>46173.72892361111</v>
+        <v>46173.20033564815</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>5.43</v>
+        <v>5.63</v>
       </c>
       <c r="L150" s="10" t="n">
-        <v>46173.81170138889</v>
+        <v>46173.26480324074</v>
       </c>
       <c r="M150" s="10" t="n">
-        <v>46173.91047453704</v>
+        <v>46173.38116898148</v>
       </c>
       <c r="N150" s="5" t="n">
-        <v>1.99</v>
+        <v>1.55</v>
       </c>
       <c r="O150" s="5" t="n">
-        <v>2.37</v>
+        <v>2.79</v>
       </c>
       <c r="P150" s="5" t="n">
-        <v>2.37</v>
+        <v>2.79</v>
       </c>
       <c r="Q150" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R150" s="5" t="n">
-        <v>9.789999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="S150" s="5" t="n">
-        <v>9.789999999999999</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="T150" s="5" t="n"/>
       <c r="U150" s="5" t="n">
@@ -27482,7 +27403,7 @@
         <v>7264</v>
       </c>
       <c r="W150" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X150" s="6" t="n">
         <v>0</v>
@@ -27511,56 +27432,56 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>71-8002 สมประสงค์ หัวลาก10W</t>
+          <t>71-8009 ชรินทร์ หัวลาก10W</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>7.28</t>
+          <t>5.28</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>8.31</t>
+          <t>5.28</t>
         </is>
       </c>
       <c r="I151" s="11" t="n">
-        <v>46172.96576388889</v>
+        <v>46172.97828703704</v>
       </c>
       <c r="J151" s="11" t="n">
-        <v>46173.20033564815</v>
+        <v>46173.5018287037</v>
       </c>
       <c r="K151" s="2" t="n">
-        <v>5.63</v>
+        <v>12.56</v>
       </c>
       <c r="L151" s="11" t="n">
-        <v>46173.26480324074</v>
+        <v>46173.57653935185</v>
       </c>
       <c r="M151" s="11" t="n">
-        <v>46173.38116898148</v>
+        <v>46173.62144675926</v>
       </c>
       <c r="N151" s="2" t="n">
-        <v>1.55</v>
+        <v>1.79</v>
       </c>
       <c r="O151" s="2" t="n">
-        <v>2.79</v>
+        <v>1.08</v>
       </c>
       <c r="P151" s="2" t="n">
-        <v>2.79</v>
+        <v>1.08</v>
       </c>
       <c r="Q151" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R151" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="S151" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="T151" s="2" t="n"/>
       <c r="U151" s="2" t="n">
@@ -27584,7 +27505,7 @@
     </row>
     <row r="152">
       <c r="A152" s="8" t="n">
-        <v>46173</v>
+        <v>46172</v>
       </c>
       <c r="B152" s="8" t="n">
         <v>46172</v>
@@ -27594,61 +27515,61 @@
       </c>
       <c r="D152" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="E152" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="F152" s="5" t="inlineStr">
         <is>
-          <t>71-8009 ชรินทร์ หัวลาก10W</t>
+          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
         </is>
       </c>
       <c r="G152" s="5" t="inlineStr">
         <is>
-          <t>5.28</t>
+          <t>2.40</t>
         </is>
       </c>
       <c r="H152" s="5" t="inlineStr">
         <is>
-          <t>5.28</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="I152" s="10" t="n">
-        <v>46172.97828703704</v>
+        <v>46172.75962962963</v>
       </c>
       <c r="J152" s="10" t="n">
-        <v>46173.5018287037</v>
+        <v>46173.02157407408</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>12.56</v>
+        <v>6.29</v>
       </c>
       <c r="L152" s="10" t="n">
-        <v>46173.57653935185</v>
+        <v>46173.09358796296</v>
       </c>
       <c r="M152" s="10" t="n">
-        <v>46173.62144675926</v>
+        <v>46173.18756944445</v>
       </c>
       <c r="N152" s="5" t="n">
-        <v>1.79</v>
+        <v>1.73</v>
       </c>
       <c r="O152" s="5" t="n">
-        <v>1.08</v>
+        <v>2.26</v>
       </c>
       <c r="P152" s="5" t="n">
-        <v>1.08</v>
+        <v>2.26</v>
       </c>
       <c r="Q152" s="5" t="n">
         <v>0</v>
       </c>
       <c r="R152" s="5" t="n">
-        <v>15.44</v>
+        <v>10.27</v>
       </c>
       <c r="S152" s="5" t="n">
-        <v>15.44</v>
+        <v>10.27</v>
       </c>
       <c r="T152" s="5" t="n"/>
       <c r="U152" s="5" t="n">
@@ -27658,7 +27579,7 @@
         <v>7264</v>
       </c>
       <c r="W152" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="X152" s="6" t="n">
         <v>0</v>
@@ -27672,10 +27593,10 @@
     </row>
     <row r="153">
       <c r="A153" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B153" s="9" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="C153" s="9" t="n">
         <v>46173</v>
@@ -27697,46 +27618,46 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
+          <t>2.41</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
           <t>2.40</t>
         </is>
       </c>
-      <c r="H153" s="2" t="inlineStr">
-        <is>
-          <t>2.39</t>
-        </is>
-      </c>
       <c r="I153" s="11" t="n">
-        <v>46172.75962962963</v>
+        <v>46173.25349537037</v>
       </c>
       <c r="J153" s="11" t="n">
-        <v>46173.02157407408</v>
+        <v>46173.31078703704</v>
       </c>
       <c r="K153" s="2" t="n">
-        <v>6.29</v>
+        <v>1.38</v>
       </c>
       <c r="L153" s="11" t="n">
-        <v>46173.09358796296</v>
+        <v>46173.385625</v>
       </c>
       <c r="M153" s="11" t="n">
-        <v>46173.18756944445</v>
+        <v>46173.41065972222</v>
       </c>
       <c r="N153" s="2" t="n">
-        <v>1.73</v>
+        <v>1.8</v>
       </c>
       <c r="O153" s="2" t="n">
-        <v>2.26</v>
+        <v>0.6</v>
       </c>
       <c r="P153" s="2" t="n">
-        <v>2.26</v>
+        <v>0.6</v>
       </c>
       <c r="Q153" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R153" s="2" t="n">
-        <v>10.27</v>
+        <v>3.77</v>
       </c>
       <c r="S153" s="2" t="n">
-        <v>10.27</v>
+        <v>3.77</v>
       </c>
       <c r="T153" s="2" t="n"/>
       <c r="U153" s="2" t="n">
@@ -27746,7 +27667,7 @@
         <v>7264</v>
       </c>
       <c r="W153" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="X153" s="7" t="n">
         <v>0</v>
@@ -27758,96 +27679,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="C154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="D154" s="5" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="E154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="F154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217 เนื้อ หัวลาก10W ตระไคร้</t>
-        </is>
-      </c>
-      <c r="G154" s="5" t="inlineStr">
-        <is>
-          <t>2.41</t>
-        </is>
-      </c>
-      <c r="H154" s="5" t="inlineStr">
-        <is>
-          <t>2.40</t>
-        </is>
-      </c>
-      <c r="I154" s="10" t="n">
-        <v>46173.25349537037</v>
-      </c>
-      <c r="J154" s="10" t="n">
-        <v>46173.31078703704</v>
-      </c>
-      <c r="K154" s="5" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="L154" s="10" t="n">
-        <v>46173.385625</v>
-      </c>
-      <c r="M154" s="10" t="n">
-        <v>46173.41065972222</v>
-      </c>
-      <c r="N154" s="5" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O154" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="P154" s="5" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q154" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R154" s="5" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="S154" s="5" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="T154" s="5" t="n"/>
-      <c r="U154" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V154" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="W154" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="X154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z154" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Z154"/>
+  <autoFilter ref="A1:Z153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27858,7 +27691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -31213,7 +31046,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C134" s="6" t="n">
@@ -31234,18 +31067,18 @@
     </row>
     <row r="135">
       <c r="A135" s="9" t="n">
-        <v>46170</v>
+        <v>46171</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C135" s="7" t="n">
         <v>7360</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>3680</v>
+        <v>0</v>
       </c>
       <c r="E135" s="7" t="n">
         <v>0</v>
@@ -31288,7 +31121,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C137" s="7" t="n">
@@ -31313,7 +31146,7 @@
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C138" s="6" t="n">
@@ -31363,7 +31196,7 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C140" s="6" t="n">
@@ -31413,11 +31246,11 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C142" s="6" t="n">
-        <v>7360</v>
+        <v>7264</v>
       </c>
       <c r="D142" s="6" t="n">
         <v>0</v>
@@ -31434,18 +31267,18 @@
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C143" s="7" t="n">
         <v>7264</v>
       </c>
       <c r="D143" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E143" s="7" t="n">
         <v>0</v>
@@ -31463,14 +31296,14 @@
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C144" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D144" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E144" s="6" t="n">
         <v>0</v>
@@ -31513,14 +31346,14 @@
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C146" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D146" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E146" s="6" t="n">
         <v>0</v>
@@ -31538,7 +31371,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C147" s="7" t="n">
@@ -31559,18 +31392,18 @@
     </row>
     <row r="148">
       <c r="A148" s="8" t="n">
-        <v>46172</v>
+        <v>46173</v>
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C148" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D148" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E148" s="6" t="n">
         <v>0</v>
@@ -31613,14 +31446,14 @@
       </c>
       <c r="B150" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C150" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D150" s="6" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E150" s="6" t="n">
         <v>0</v>
@@ -31638,7 +31471,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C151" s="7" t="n">
@@ -31663,14 +31496,14 @@
       </c>
       <c r="B152" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C152" s="6" t="n">
         <v>7264</v>
       </c>
       <c r="D152" s="6" t="n">
-        <v>3632</v>
+        <v>0</v>
       </c>
       <c r="E152" s="6" t="n">
         <v>0</v>
@@ -31695,7 +31528,7 @@
         <v>7264</v>
       </c>
       <c r="D153" s="7" t="n">
-        <v>0</v>
+        <v>3632</v>
       </c>
       <c r="E153" s="7" t="n">
         <v>0</v>
@@ -31707,33 +31540,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="8" t="n">
-        <v>46173</v>
-      </c>
-      <c r="B154" s="5" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C154" s="6" t="n">
-        <v>7264</v>
-      </c>
-      <c r="D154" s="6" t="n">
-        <v>3632</v>
-      </c>
-      <c r="E154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F154" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G154" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G154"/>
+  <autoFilter ref="A1:G153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33364,22 +33172,22 @@
         <v>46170</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D29" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D29" s="2" t="n">
-        <v>10</v>
-      </c>
       <c r="E29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H29" s="2" t="n">
         <v>1</v>
@@ -33487,7 +33295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -38421,25 +38229,25 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>18.85</v>
+        <v>16.5</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>3.68</v>
+        <v>3.28</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>1.56</v>
+        <v>11.61</v>
       </c>
       <c r="G105" s="2" t="n">
-        <v>13.61</v>
+        <v>1.61</v>
       </c>
       <c r="H105" s="2" t="n">
         <v>0</v>
@@ -38448,45 +38256,45 @@
         <v>0</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>3.68</v>
+        <v>3.28</v>
       </c>
       <c r="K105" s="2" t="n">
-        <v>1.56</v>
+        <v>11.61</v>
       </c>
       <c r="L105" s="2" t="n">
-        <v>18.85</v>
+        <v>16.5</v>
       </c>
       <c r="M105" s="2" t="n">
-        <v>5.15</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D106" s="5" t="n">
-        <v>16.5</v>
+        <v>18.35</v>
       </c>
       <c r="E106" s="5" t="n">
-        <v>3.28</v>
+        <v>5.44</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>11.61</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="G106" s="5" t="n">
-        <v>1.61</v>
+        <v>3.96</v>
       </c>
       <c r="H106" s="5" t="n">
         <v>0</v>
@@ -38495,16 +38303,16 @@
         <v>0</v>
       </c>
       <c r="J106" s="5" t="n">
-        <v>3.28</v>
+        <v>5.44</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>11.61</v>
+        <v>8.949999999999999</v>
       </c>
       <c r="L106" s="5" t="n">
-        <v>16.5</v>
+        <v>18.35</v>
       </c>
       <c r="M106" s="5" t="n">
-        <v>7.5</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="107">
@@ -38515,7 +38323,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -38524,16 +38332,16 @@
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>18.35</v>
+        <v>18.22</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>5.44</v>
+        <v>7.66</v>
       </c>
       <c r="F107" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>7.12</v>
       </c>
       <c r="G107" s="2" t="n">
-        <v>3.96</v>
+        <v>3.44</v>
       </c>
       <c r="H107" s="2" t="n">
         <v>0</v>
@@ -38542,16 +38350,16 @@
         <v>0</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>5.44</v>
+        <v>7.66</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>7.12</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>18.35</v>
+        <v>18.22</v>
       </c>
       <c r="M107" s="2" t="n">
-        <v>5.65</v>
+        <v>5.78</v>
       </c>
     </row>
     <row r="108">
@@ -38562,7 +38370,7 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
@@ -38571,16 +38379,16 @@
         </is>
       </c>
       <c r="D108" s="5" t="n">
-        <v>18.22</v>
+        <v>21.08</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>7.66</v>
+        <v>8.5</v>
       </c>
       <c r="F108" s="5" t="n">
-        <v>7.12</v>
+        <v>8.01</v>
       </c>
       <c r="G108" s="5" t="n">
-        <v>3.44</v>
+        <v>4.57</v>
       </c>
       <c r="H108" s="5" t="n">
         <v>0</v>
@@ -38589,16 +38397,16 @@
         <v>0</v>
       </c>
       <c r="J108" s="5" t="n">
-        <v>7.66</v>
+        <v>8.5</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>7.12</v>
+        <v>8.01</v>
       </c>
       <c r="L108" s="5" t="n">
-        <v>18.22</v>
+        <v>21.08</v>
       </c>
       <c r="M108" s="5" t="n">
-        <v>5.78</v>
+        <v>2.92</v>
       </c>
     </row>
     <row r="109">
@@ -38609,7 +38417,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -38618,16 +38426,16 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>21.08</v>
+        <v>19.32</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>8.5</v>
+        <v>12.75</v>
       </c>
       <c r="F109" s="2" t="n">
-        <v>8.01</v>
+        <v>2.68</v>
       </c>
       <c r="G109" s="2" t="n">
-        <v>4.57</v>
+        <v>3.9</v>
       </c>
       <c r="H109" s="2" t="n">
         <v>0</v>
@@ -38636,16 +38444,16 @@
         <v>0</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>8.5</v>
+        <v>12.75</v>
       </c>
       <c r="K109" s="2" t="n">
-        <v>8.01</v>
+        <v>2.68</v>
       </c>
       <c r="L109" s="2" t="n">
-        <v>21.08</v>
+        <v>19.32</v>
       </c>
       <c r="M109" s="2" t="n">
-        <v>2.92</v>
+        <v>4.68</v>
       </c>
     </row>
     <row r="110">
@@ -38656,25 +38464,25 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D110" s="5" t="n">
-        <v>19.32</v>
+        <v>17.35</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>12.75</v>
+        <v>7.33</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>2.68</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>3.9</v>
+        <v>1.63</v>
       </c>
       <c r="H110" s="5" t="n">
         <v>0</v>
@@ -38683,45 +38491,45 @@
         <v>0</v>
       </c>
       <c r="J110" s="5" t="n">
-        <v>12.75</v>
+        <v>7.33</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>2.68</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="L110" s="5" t="n">
-        <v>19.32</v>
+        <v>17.35</v>
       </c>
       <c r="M110" s="5" t="n">
-        <v>4.68</v>
+        <v>6.65</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>17.35</v>
+        <v>11.92</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>7.33</v>
+        <v>3.66</v>
       </c>
       <c r="F111" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>6.14</v>
       </c>
       <c r="G111" s="2" t="n">
-        <v>1.63</v>
+        <v>2.13</v>
       </c>
       <c r="H111" s="2" t="n">
         <v>0</v>
@@ -38730,16 +38538,16 @@
         <v>0</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>7.33</v>
+        <v>3.66</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>6.14</v>
       </c>
       <c r="L111" s="2" t="n">
-        <v>17.35</v>
+        <v>11.92</v>
       </c>
       <c r="M111" s="2" t="n">
-        <v>6.65</v>
+        <v>12.08</v>
       </c>
     </row>
     <row r="112">
@@ -38750,7 +38558,7 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
@@ -38759,16 +38567,16 @@
         </is>
       </c>
       <c r="D112" s="5" t="n">
-        <v>11.92</v>
+        <v>23.52</v>
       </c>
       <c r="E112" s="5" t="n">
-        <v>3.66</v>
+        <v>4.75</v>
       </c>
       <c r="F112" s="5" t="n">
-        <v>6.14</v>
+        <v>7.66</v>
       </c>
       <c r="G112" s="5" t="n">
-        <v>2.13</v>
+        <v>11.11</v>
       </c>
       <c r="H112" s="5" t="n">
         <v>0</v>
@@ -38777,16 +38585,16 @@
         <v>0</v>
       </c>
       <c r="J112" s="5" t="n">
-        <v>3.66</v>
+        <v>4.75</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>6.14</v>
+        <v>7.66</v>
       </c>
       <c r="L112" s="5" t="n">
-        <v>11.92</v>
+        <v>23.52</v>
       </c>
       <c r="M112" s="5" t="n">
-        <v>12.08</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="113">
@@ -38797,7 +38605,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -38806,34 +38614,34 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>23.52</v>
+        <v>11.07</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>4.75</v>
+        <v>6.13</v>
       </c>
       <c r="F113" s="2" t="n">
-        <v>7.66</v>
+        <v>3.05</v>
       </c>
       <c r="G113" s="2" t="n">
-        <v>11.11</v>
+        <v>1.89</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>0</v>
+        <v>0.53</v>
       </c>
       <c r="I113" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>4.75</v>
+        <v>6.65</v>
       </c>
       <c r="K113" s="2" t="n">
-        <v>7.66</v>
+        <v>3.05</v>
       </c>
       <c r="L113" s="2" t="n">
-        <v>23.52</v>
+        <v>11.6</v>
       </c>
       <c r="M113" s="2" t="n">
-        <v>0.48</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="114">
@@ -38844,7 +38652,7 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
@@ -38853,34 +38661,34 @@
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>11.07</v>
+        <v>15.05</v>
       </c>
       <c r="E114" s="5" t="n">
-        <v>6.13</v>
+        <v>6.97</v>
       </c>
       <c r="F114" s="5" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="G114" s="5" t="n">
-        <v>1.89</v>
+        <v>2.97</v>
       </c>
       <c r="H114" s="5" t="n">
-        <v>0.53</v>
+        <v>0</v>
       </c>
       <c r="I114" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J114" s="5" t="n">
-        <v>6.65</v>
+        <v>6.97</v>
       </c>
       <c r="K114" s="5" t="n">
-        <v>3.05</v>
+        <v>5.11</v>
       </c>
       <c r="L114" s="5" t="n">
-        <v>11.6</v>
+        <v>15.05</v>
       </c>
       <c r="M114" s="5" t="n">
-        <v>12.4</v>
+        <v>8.949999999999999</v>
       </c>
     </row>
     <row r="115">
@@ -38891,25 +38699,25 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>15.05</v>
+        <v>32.17</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>6.97</v>
+        <v>9.98</v>
       </c>
       <c r="F115" s="2" t="n">
-        <v>5.11</v>
+        <v>18.74</v>
       </c>
       <c r="G115" s="2" t="n">
-        <v>2.97</v>
+        <v>3.44</v>
       </c>
       <c r="H115" s="2" t="n">
         <v>0</v>
@@ -38918,63 +38726,63 @@
         <v>0</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>6.97</v>
+        <v>9.98</v>
       </c>
       <c r="K115" s="2" t="n">
-        <v>5.11</v>
+        <v>18.74</v>
       </c>
       <c r="L115" s="2" t="n">
-        <v>15.05</v>
+        <v>32.17</v>
       </c>
       <c r="M115" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>-8.17</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>72-1217</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>LCB</t>
+          <t>BigC</t>
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>32.17</v>
+        <v>20.31</v>
       </c>
       <c r="E116" s="5" t="n">
-        <v>9.98</v>
+        <v>12.79</v>
       </c>
       <c r="F116" s="5" t="n">
-        <v>18.74</v>
+        <v>3.44</v>
       </c>
       <c r="G116" s="5" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="H116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I116" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J116" s="5" t="n">
+        <v>12.79</v>
+      </c>
+      <c r="K116" s="5" t="n">
         <v>3.44</v>
       </c>
-      <c r="H116" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I116" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J116" s="5" t="n">
-        <v>9.98</v>
-      </c>
-      <c r="K116" s="5" t="n">
-        <v>18.74</v>
-      </c>
       <c r="L116" s="5" t="n">
-        <v>32.17</v>
+        <v>20.31</v>
       </c>
       <c r="M116" s="5" t="n">
-        <v>-8.17</v>
+        <v>3.69</v>
       </c>
     </row>
     <row r="117">
@@ -38985,7 +38793,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -38994,34 +38802,34 @@
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>20.31</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>12.79</v>
+        <v>5.63</v>
       </c>
       <c r="F117" s="2" t="n">
-        <v>3.44</v>
+        <v>2.79</v>
       </c>
       <c r="G117" s="2" t="n">
-        <v>4.07</v>
+        <v>1.55</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>0</v>
+        <v>13.11</v>
       </c>
       <c r="I117" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>12.79</v>
+        <v>18.73</v>
       </c>
       <c r="K117" s="2" t="n">
-        <v>3.44</v>
+        <v>2.79</v>
       </c>
       <c r="L117" s="2" t="n">
-        <v>20.31</v>
+        <v>23.07</v>
       </c>
       <c r="M117" s="2" t="n">
-        <v>3.69</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="118">
@@ -39032,7 +38840,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -39041,34 +38849,34 @@
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>9.970000000000001</v>
+        <v>0</v>
       </c>
       <c r="E118" s="5" t="n">
-        <v>5.63</v>
+        <v>0</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>2.79</v>
+        <v>0</v>
       </c>
       <c r="G118" s="5" t="n">
-        <v>1.55</v>
+        <v>0</v>
       </c>
       <c r="H118" s="5" t="n">
-        <v>13.11</v>
+        <v>0.61</v>
       </c>
       <c r="I118" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J118" s="5" t="n">
-        <v>18.73</v>
+        <v>0.61</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>2.79</v>
+        <v>0</v>
       </c>
       <c r="L118" s="5" t="n">
-        <v>23.07</v>
+        <v>0.61</v>
       </c>
       <c r="M118" s="5" t="n">
-        <v>0.93</v>
+        <v>23.39</v>
       </c>
     </row>
     <row r="119">
@@ -39079,7 +38887,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -39088,34 +38896,34 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>0</v>
+        <v>15.44</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0</v>
+        <v>12.56</v>
       </c>
       <c r="F119" s="2" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="G119" s="2" t="n">
-        <v>0</v>
+        <v>1.79</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>0.61</v>
+        <v>0</v>
       </c>
       <c r="I119" s="2" t="n">
         <v>0</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.61</v>
+        <v>12.56</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>0</v>
+        <v>1.08</v>
       </c>
       <c r="L119" s="2" t="n">
-        <v>0.61</v>
+        <v>15.44</v>
       </c>
       <c r="M119" s="2" t="n">
-        <v>23.39</v>
+        <v>8.56</v>
       </c>
     </row>
     <row r="120">
@@ -39126,94 +38934,47 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>72-1217</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>BigC</t>
+          <t>LCB</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
-        <v>15.44</v>
+        <v>3.77</v>
       </c>
       <c r="E120" s="5" t="n">
-        <v>12.56</v>
+        <v>1.38</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>1.08</v>
+        <v>0.6</v>
       </c>
       <c r="G120" s="5" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="H120" s="5" t="n">
-        <v>0</v>
+        <v>5.35</v>
       </c>
       <c r="I120" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J120" s="5" t="n">
-        <v>12.56</v>
+        <v>6.72</v>
       </c>
       <c r="K120" s="5" t="n">
-        <v>1.08</v>
+        <v>0.6</v>
       </c>
       <c r="L120" s="5" t="n">
-        <v>15.44</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="M120" s="5" t="n">
-        <v>8.56</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-31</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
-        <is>
-          <t>72-1217</t>
-        </is>
-      </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>LCB</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="n">
-        <v>3.77</v>
-      </c>
-      <c r="E121" s="2" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="F121" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G121" s="2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="H121" s="2" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="I121" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J121" s="2" t="n">
-        <v>6.72</v>
-      </c>
-      <c r="K121" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="L121" s="2" t="n">
-        <v>9.119999999999999</v>
-      </c>
-      <c r="M121" s="2" t="n">
         <v>14.88</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M121"/>
+  <autoFilter ref="A1:M120"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Oatside July: split manual-trip 25% surcharge into its own column (grand unchanged 1,537,168)
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -34,7 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$143</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$143</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04 14:33</t>
+          <t>2026-08-04 16:11</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1255128</v>
+        <v>1251712</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>24056</v>
+        <v>20640</v>
       </c>
     </row>
     <row r="15">
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>197288</v>
+        <v>200704</v>
       </c>
     </row>
     <row r="21">
@@ -1412,10 +1412,10 @@
         <v>6976</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>8720</v>
+        <v>6976</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>0</v>
+        <v>1744</v>
       </c>
       <c r="H18" s="6" t="n">
         <v>0</v>
@@ -2336,10 +2336,10 @@
         <v>6688</v>
       </c>
       <c r="F46" s="6" t="n">
-        <v>8360</v>
+        <v>6688</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>0</v>
+        <v>1672</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>0</v>
@@ -5561,7 +5561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5571,7 +5571,7 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
@@ -6024,7 +6024,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8004</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -6034,19 +6034,27 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>override_include</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>include_50</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>วันนี้มีเที่ยวจริง 1 เที่ยว (TO-OTL15906 — GPS ทำขาส่งหาย engine เห็น 0 เที่ยว) → เก็บส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% ตามปกติ; ตัวเที่ยวอยู่ใน manual_extra_trips</t>
+        </is>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
           <t>2026-07-04</t>
@@ -6062,11 +6070,11 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>46209</v>
+        <v>46207</v>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -6091,7 +6099,7 @@
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr"/>
@@ -6108,7 +6116,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -6146,11 +6154,11 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>46210</v>
+        <v>46209</v>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -6175,7 +6183,7 @@
       <c r="H14" s="5" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr"/>
@@ -6192,7 +6200,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -6234,7 +6242,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -6276,7 +6284,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -6318,7 +6326,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -6356,11 +6364,11 @@
     </row>
     <row r="19">
       <c r="A19" s="9" t="n">
-        <v>46211</v>
+        <v>46210</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -6370,11 +6378,11 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -6385,15 +6393,15 @@
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>6688</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="20">
@@ -6402,7 +6410,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -6412,11 +6420,11 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -6435,7 +6443,7 @@
         <v>6688</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>1672</v>
+        <v>6688</v>
       </c>
     </row>
     <row r="21">
@@ -6444,7 +6452,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -6486,7 +6494,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -6528,7 +6536,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -6566,11 +6574,11 @@
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>46212</v>
+        <v>46211</v>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -6595,7 +6603,7 @@
       <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr"/>
@@ -6612,7 +6620,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -6650,11 +6658,11 @@
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>71-5041</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -6679,7 +6687,7 @@
       <c r="H26" s="5" t="inlineStr"/>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
@@ -6696,7 +6704,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -6738,7 +6746,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -6776,11 +6784,11 @@
     </row>
     <row r="29">
       <c r="A29" s="9" t="n">
-        <v>46215</v>
+        <v>46213</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -6805,7 +6813,7 @@
       <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
@@ -6818,11 +6826,11 @@
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>46215</v>
+        <v>46214</v>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5041</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -6832,22 +6840,30 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>override_include</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>include_50</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>วันนี้มีเที่ยวจริง 1 เที่ยว (TO-OTL16400 — GPS ทำขาส่งหาย engine เห็น 0 เที่ยว) → เก็บส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% ตามปกติแทน no_finish 100% ที่ลั่นผิด; ตัวเที่ยวอยู่ใน manual_extra_trips</t>
+        </is>
+      </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
@@ -6860,7 +6876,7 @@
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -6889,7 +6905,7 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
@@ -6902,11 +6918,11 @@
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>46216</v>
+        <v>46215</v>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -6931,7 +6947,7 @@
       <c r="H32" s="5" t="inlineStr"/>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr"/>
@@ -6948,7 +6964,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -6990,7 +7006,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -7028,11 +7044,11 @@
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7057,7 +7073,7 @@
       <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
@@ -7070,11 +7086,11 @@
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -7099,7 +7115,7 @@
       <c r="H36" s="5" t="inlineStr"/>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
@@ -7116,7 +7132,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -7158,7 +7174,7 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -7196,11 +7212,11 @@
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
-        <v>46218</v>
+        <v>46217</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -7225,7 +7241,7 @@
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
@@ -7238,11 +7254,11 @@
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>46218</v>
+        <v>46217</v>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -7267,7 +7283,7 @@
       <c r="H40" s="5" t="inlineStr"/>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
@@ -7284,7 +7300,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7322,11 +7338,11 @@
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -7351,7 +7367,7 @@
       <c r="H42" s="5" t="inlineStr"/>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr"/>
@@ -7364,11 +7380,11 @@
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
-        <v>46219</v>
+        <v>46218</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -7378,11 +7394,11 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -7393,7 +7409,7 @@
       <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
@@ -7401,7 +7417,7 @@
         <v>6688</v>
       </c>
       <c r="L43" s="7" t="n">
-        <v>6688</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="44">
@@ -7410,7 +7426,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
@@ -7452,7 +7468,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -7462,11 +7478,11 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -7485,16 +7501,16 @@
         <v>6688</v>
       </c>
       <c r="L45" s="7" t="n">
-        <v>1672</v>
+        <v>6688</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -7519,7 +7535,7 @@
       <c r="H46" s="5" t="inlineStr"/>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
@@ -7532,11 +7548,11 @@
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>46220</v>
+        <v>46219</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -7561,7 +7577,7 @@
       <c r="H47" s="2" t="inlineStr"/>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
@@ -7578,7 +7594,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -7620,7 +7636,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -7630,11 +7646,11 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -7653,16 +7669,16 @@
         <v>6688</v>
       </c>
       <c r="L49" s="7" t="n">
-        <v>6688</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
@@ -7687,7 +7703,7 @@
       <c r="H50" s="5" t="inlineStr"/>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr"/>
@@ -7700,11 +7716,11 @@
     </row>
     <row r="51">
       <c r="A51" s="9" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -7714,11 +7730,11 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -7729,7 +7745,7 @@
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
@@ -7737,16 +7753,16 @@
         <v>6688</v>
       </c>
       <c r="L51" s="7" t="n">
-        <v>1672</v>
+        <v>6688</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>46222</v>
+        <v>46221</v>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -7771,7 +7787,7 @@
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr"/>
@@ -7784,7 +7800,7 @@
     </row>
     <row r="53">
       <c r="A53" s="9" t="n">
-        <v>46223</v>
+        <v>46221</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
@@ -7813,7 +7829,7 @@
       <c r="H53" s="2" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -7826,11 +7842,11 @@
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -7855,7 +7871,7 @@
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr"/>
@@ -7872,7 +7888,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -7914,7 +7930,7 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
@@ -7952,11 +7968,11 @@
     </row>
     <row r="57">
       <c r="A57" s="9" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -7981,7 +7997,7 @@
       <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
@@ -7994,11 +8010,11 @@
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -8023,7 +8039,7 @@
       <c r="H58" s="5" t="inlineStr"/>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr"/>
@@ -8040,7 +8056,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -8082,7 +8098,7 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -8092,11 +8108,11 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
@@ -8115,16 +8131,16 @@
         <v>6688</v>
       </c>
       <c r="L60" s="6" t="n">
-        <v>6688</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -8149,24 +8165,24 @@
       <c r="H61" s="2" t="inlineStr"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="7" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="L61" s="7" t="n">
-        <v>1696</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -8176,11 +8192,11 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
@@ -8191,20 +8207,20 @@
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr"/>
       <c r="K62" s="6" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="L62" s="6" t="n">
-        <v>1696</v>
+        <v>6688</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
@@ -8233,20 +8249,20 @@
       <c r="H63" s="2" t="inlineStr"/>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="L63" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>46226</v>
+        <v>46225</v>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
@@ -8275,15 +8291,15 @@
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr"/>
       <c r="K64" s="6" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="L64" s="6" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="65">
@@ -8292,7 +8308,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -8302,11 +8318,11 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -8325,16 +8341,16 @@
         <v>6880</v>
       </c>
       <c r="L65" s="7" t="n">
-        <v>6880</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -8359,7 +8375,7 @@
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="J66" s="5" t="inlineStr"/>
@@ -8372,11 +8388,11 @@
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
-        <v>46227</v>
+        <v>46226</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -8401,7 +8417,7 @@
       <c r="H67" s="2" t="inlineStr"/>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
@@ -8418,7 +8434,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -8460,7 +8476,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -8502,7 +8518,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
@@ -8540,11 +8556,11 @@
     </row>
     <row r="71">
       <c r="A71" s="9" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -8554,11 +8570,11 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -8569,7 +8585,7 @@
       <c r="H71" s="2" t="inlineStr"/>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
@@ -8577,16 +8593,16 @@
         <v>6880</v>
       </c>
       <c r="L71" s="7" t="n">
-        <v>1720</v>
+        <v>6880</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>46228</v>
+        <v>46227</v>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -8611,7 +8627,7 @@
       <c r="H72" s="5" t="inlineStr"/>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J72" s="5" t="inlineStr"/>
@@ -8628,7 +8644,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -8670,7 +8686,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -8712,7 +8728,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -8750,11 +8766,11 @@
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>46229</v>
+        <v>46228</v>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -8764,11 +8780,11 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
@@ -8779,7 +8795,7 @@
       <c r="H76" s="5" t="inlineStr"/>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="J76" s="5" t="inlineStr"/>
@@ -8787,12 +8803,12 @@
         <v>6880</v>
       </c>
       <c r="L76" s="6" t="n">
-        <v>6880</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="n">
-        <v>46229</v>
+        <v>46228</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -8821,7 +8837,7 @@
       <c r="H77" s="2" t="inlineStr"/>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
@@ -8834,11 +8850,11 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -8848,11 +8864,11 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -8863,7 +8879,7 @@
       <c r="H78" s="5" t="inlineStr"/>
       <c r="I78" s="5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="J78" s="5" t="inlineStr"/>
@@ -8871,16 +8887,16 @@
         <v>6880</v>
       </c>
       <c r="L78" s="6" t="n">
-        <v>1720</v>
+        <v>6880</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8905,7 +8921,7 @@
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
@@ -8922,7 +8938,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -8960,11 +8976,11 @@
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
-        <v>46232</v>
+        <v>46230</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -8989,7 +9005,7 @@
       <c r="H81" s="2" t="inlineStr"/>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
@@ -9002,11 +9018,11 @@
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>46232</v>
+        <v>46230</v>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -9031,7 +9047,7 @@
       <c r="H82" s="5" t="inlineStr"/>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr"/>
@@ -9048,7 +9064,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -9086,11 +9102,11 @@
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -9115,7 +9131,7 @@
       <c r="H84" s="5" t="inlineStr"/>
       <c r="I84" s="5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="J84" s="5" t="inlineStr"/>
@@ -9128,11 +9144,11 @@
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -9157,7 +9173,7 @@
       <c r="H85" s="2" t="inlineStr"/>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -9174,7 +9190,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -9216,7 +9232,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -9258,7 +9274,7 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -9296,11 +9312,11 @@
     </row>
     <row r="89">
       <c r="A89" s="9" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -9325,7 +9341,7 @@
       <c r="H89" s="2" t="inlineStr"/>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
@@ -9338,11 +9354,11 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -9367,7 +9383,7 @@
       <c r="H90" s="5" t="inlineStr"/>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr"/>
@@ -9384,7 +9400,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -9426,7 +9442,7 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -9468,7 +9484,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -9504,8 +9520,92 @@
         <v>1720</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="8" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>71-8003</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>BigC</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>one_trip_billed_day</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr"/>
+      <c r="H94" s="5" t="inlineStr"/>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr"/>
+      <c r="K94" s="6" t="n">
+        <v>6880</v>
+      </c>
+      <c r="L94" s="6" t="n">
+        <v>1720</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="9" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>BigC</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>one_trip_billed_day</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="7" t="n">
+        <v>6880</v>
+      </c>
+      <c r="L95" s="7" t="n">
+        <v>1720</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L93"/>
+  <autoFilter ref="A1:L95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9575,11 +9675,11 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>8720</v>
+        <v>6976</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>เดลี่ AYU 4/7 TO-OTL15906 (อุดมชัย) — GPS มีขาต้นทาง 2/7 11:23→4/7 10:45 (47ชม.) แต่ขา P&amp;G หาย; เที่ยวจริงตามใบงาน = เรท 4/7 6,976 + ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% 1,744 (วันนั้น 8004 วิ่งเที่ยวเดียว)</t>
+          <t>เดลี่ AYU 4/7 TO-OTL15906 (อุดมชัย) — GPS มีขาต้นทาง 2/7 11:23→4/7 10:45 (47ชม.) แต่ขา P&amp;G หาย; เที่ยวจริงตามใบงาน @เรท 4/7 (ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% เก็บผ่าน override include_50 แยกช่องเหมือนเที่ยวปกติ)</t>
         </is>
       </c>
     </row>
@@ -9593,11 +9693,11 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>8360</v>
+        <v>6688</v>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>เดลี่ AYU 11/7 TO-OTL16400 — GPS มีขาต้นทาง 10/7 22:34→11/7 04:40 แต่ขา P&amp;G หาย; เที่ยวที่ 5 ของ 5041 ตามใบงาน = เรท 11/7 6,688 + ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% 1,672 (คู่ exclude_50 กัน no_finish 100% ลั่น)</t>
+          <t>เดลี่ AYU 11/7 TO-OTL16400 — GPS มีขาต้นทาง 10/7 22:34→11/7 04:40 แต่ขา P&amp;G หาย; เที่ยวที่ 5 ของ 5041 ตามใบงาน @เรท 11/7 (override include_50 เก็บ 25% แยกช่อง + กัน no_finish 100% ลั่น)</t>
         </is>
       </c>
     </row>
@@ -10314,7 +10414,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1255128</v>
+        <v>1251712</v>
       </c>
     </row>
     <row r="3">
@@ -10329,7 +10429,7 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>24056</v>
+        <v>20640</v>
       </c>
     </row>
     <row r="4">
@@ -10374,7 +10474,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>197288</v>
+        <v>200704</v>
       </c>
     </row>
     <row r="7">
@@ -11645,10 +11745,10 @@
         <v>6976</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>8720</v>
+        <v>6976</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0</v>
+        <v>1744</v>
       </c>
       <c r="H22" s="6" t="n">
         <v>0</v>
@@ -11658,7 +11758,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>ไม่เก็บ — รถแช่ต้นทาง 10.8 ชม. (รอคิว/โหลดของ ไม่ใช่ติดค้างปลายทาง) | เที่ยวเพิ่ม (ไม่มีใน GPS): เดลี่ AYU 4/7 TO-OTL15906 (อุดมชัย) — GPS มีขาต้นทาง 2/7 11:23→4/7 10:45 (47ชม.) แต่ขา P&amp;G หาย; เที่ยวจริงตามใบงาน = เรท 4/7 6,976 + ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% 1,744 (วันนั้น 8004 วิ่งเที่ยวเดียว) (+8,720.00฿)</t>
+          <t>ไม่เก็บ — รถแช่ต้นทาง 10.8 ชม. (รอคิว/โหลดของ ไม่ใช่ติดค้างปลายทาง) | เที่ยวเพิ่ม (ไม่มีใน GPS): เดลี่ AYU 4/7 TO-OTL15906 (อุดมชัย) — GPS มีขาต้นทาง 2/7 11:23→4/7 10:45 (47ชม.) แต่ขา P&amp;G หาย; เที่ยวจริงตามใบงาน @เรท 4/7 (ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% เก็บผ่าน override include_50 แยกช่องเหมือนเที่ยวปกติ) (+6,976.00฿)</t>
         </is>
       </c>
     </row>
@@ -12823,10 +12923,10 @@
         <v>6688</v>
       </c>
       <c r="F53" s="7" t="n">
-        <v>8360</v>
+        <v>6688</v>
       </c>
       <c r="G53" s="7" t="n">
-        <v>0</v>
+        <v>1672</v>
       </c>
       <c r="H53" s="7" t="n">
         <v>0</v>
@@ -12836,7 +12936,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>ไม่เก็บ [override: exclude_50] — วันนี้มีเที่ยวจริง 1 เที่ยว (TO-OTL16400) แต่ GPS ทำขาส่งหาย engine จึงเห็น 0 เที่ยวแล้วเก็บ no_finish 100% ผิด — ตัดทิ้ง; ตัวเที่ยว+ส่วนเพิ่ม 25% เก็บผ่าน manual_extra_trips แทน | เที่ยวเพิ่ม (ไม่มีใน GPS): เดลี่ AYU 11/7 TO-OTL16400 — GPS มีขาต้นทาง 10/7 22:34→11/7 04:40 แต่ขา P&amp;G หาย; เที่ยวที่ 5 ของ 5041 ตามใบงาน = เรท 11/7 6,688 + ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% 1,672 (คู่ exclude_50 กัน no_finish 100% ลั่น) (+8,360.00฿)</t>
+          <t>เก็บ 100% = 1 เรทเต็ม (รถ standby ระหว่างเที่ยว (เข้าต้นทาง 4.7 ชม. ไม่จบเที่ยว)) | เที่ยวเพิ่ม (ไม่มีใน GPS): เดลี่ AYU 11/7 TO-OTL16400 — GPS มีขาต้นทาง 10/7 22:34→11/7 04:40 แต่ขา P&amp;G หาย; เที่ยวที่ 5 ของ 5041 ตามใบงาน @เรท 11/7 (override include_50 เก็บ 25% แยกช่อง + กัน no_finish 100% ลั่น) (+6,688.00฿)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oatside July: cut Laem Chabang (WH-LCB) work from bill - remove 8001 26/7 no_finish + 5 LCB TOs (grand 1,530,288)
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -33,8 +33,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$143</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$143</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04 16:11</t>
+          <t>2026-08-05 14:34</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>200704</v>
+        <v>193824</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1537168</v>
+        <v>1530288</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I143"/>
+  <dimension ref="A1:I142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -4706,22 +4706,22 @@
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E118" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F118" s="6" t="n">
-        <v>0</v>
+        <v>13760</v>
       </c>
       <c r="G118" s="6" t="n">
-        <v>6880</v>
+        <v>0</v>
       </c>
       <c r="H118" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I118" s="6" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="119">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -4739,31 +4739,31 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E119" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F119" s="7" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I119" s="7" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
@@ -4784,10 +4784,10 @@
         <v>1720</v>
       </c>
       <c r="H120" s="6" t="n">
-        <v>0</v>
+        <v>3440</v>
       </c>
       <c r="I120" s="6" t="n">
-        <v>8600</v>
+        <v>12040</v>
       </c>
     </row>
     <row r="121">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -4817,10 +4817,10 @@
         <v>1720</v>
       </c>
       <c r="H121" s="7" t="n">
-        <v>3440</v>
+        <v>0</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>12040</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="122">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -4838,22 +4838,22 @@
         </is>
       </c>
       <c r="D122" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E122" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F122" s="6" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G122" s="6" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H122" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I122" s="6" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="123">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -4871,31 +4871,31 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E123" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F123" s="7" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I123" s="7" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
@@ -4904,22 +4904,22 @@
         </is>
       </c>
       <c r="D124" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E124" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F124" s="6" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G124" s="6" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H124" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I124" s="6" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="125">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -5003,13 +5003,13 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E127" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F127" s="7" t="n">
-        <v>13760</v>
+        <v>20640</v>
       </c>
       <c r="G127" s="7" t="n">
         <v>0</v>
@@ -5018,16 +5018,16 @@
         <v>0</v>
       </c>
       <c r="I127" s="7" t="n">
-        <v>13760</v>
+        <v>20640</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -5036,22 +5036,22 @@
         </is>
       </c>
       <c r="D128" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E128" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F128" s="6" t="n">
-        <v>20640</v>
+        <v>6880</v>
       </c>
       <c r="G128" s="6" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H128" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I128" s="6" t="n">
-        <v>20640</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="129">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -5069,22 +5069,22 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E129" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F129" s="7" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G129" s="7" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H129" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I129" s="7" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="130">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -5135,22 +5135,22 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E131" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F131" s="7" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I131" s="7" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="132">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -5188,11 +5188,11 @@
     </row>
     <row r="133">
       <c r="A133" s="9" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -5353,11 +5353,11 @@
     </row>
     <row r="138">
       <c r="A138" s="8" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -5411,10 +5411,10 @@
         <v>1720</v>
       </c>
       <c r="H139" s="7" t="n">
-        <v>0</v>
+        <v>3440</v>
       </c>
       <c r="I139" s="7" t="n">
-        <v>8600</v>
+        <v>12040</v>
       </c>
     </row>
     <row r="140">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
@@ -5444,10 +5444,10 @@
         <v>1720</v>
       </c>
       <c r="H140" s="6" t="n">
-        <v>3440</v>
+        <v>0</v>
       </c>
       <c r="I140" s="6" t="n">
-        <v>12040</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="141">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
@@ -5516,41 +5516,8 @@
         <v>8600</v>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="9" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
-        <is>
-          <t>71-8009</t>
-        </is>
-      </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E143" s="7" t="n">
-        <v>6880</v>
-      </c>
-      <c r="F143" s="7" t="n">
-        <v>6880</v>
-      </c>
-      <c r="G143" s="7" t="n">
-        <v>1720</v>
-      </c>
-      <c r="H143" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I143" s="7" t="n">
-        <v>8600</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I143"/>
+  <autoFilter ref="A1:I142"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5561,7 +5528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8854,7 +8821,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -8864,11 +8831,11 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>no_finish_day</t>
+          <t>one_trip_billed_day</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -8887,16 +8854,16 @@
         <v>6880</v>
       </c>
       <c r="L78" s="6" t="n">
-        <v>6880</v>
+        <v>1720</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8921,7 +8888,7 @@
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
@@ -8938,7 +8905,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -8980,7 +8947,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -9018,11 +8985,11 @@
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -9047,7 +9014,7 @@
       <c r="H82" s="5" t="inlineStr"/>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr"/>
@@ -9064,7 +9031,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -9106,7 +9073,7 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -9144,11 +9111,11 @@
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -9173,7 +9140,7 @@
       <c r="H85" s="2" t="inlineStr"/>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -9190,7 +9157,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -9232,7 +9199,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -9274,7 +9241,7 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -9316,7 +9283,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -9354,11 +9321,11 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -9383,7 +9350,7 @@
       <c r="H90" s="5" t="inlineStr"/>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr"/>
@@ -9400,7 +9367,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -9442,7 +9409,7 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -9484,7 +9451,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -9526,7 +9493,7 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -9562,50 +9529,8 @@
         <v>1720</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="9" t="n">
-        <v>46234</v>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>71-8009</t>
-        </is>
-      </c>
-      <c r="C95" s="2" t="inlineStr">
-        <is>
-          <t>BigC</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>one_trip_billed_day</t>
-        </is>
-      </c>
-      <c r="E95" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G95" s="2" t="inlineStr"/>
-      <c r="H95" s="2" t="inlineStr"/>
-      <c r="I95" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="J95" s="2" t="inlineStr"/>
-      <c r="K95" s="7" t="n">
-        <v>6880</v>
-      </c>
-      <c r="L95" s="7" t="n">
-        <v>1720</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L95"/>
+  <autoFilter ref="A1:L94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10474,7 +10399,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>200704</v>
+        <v>193824</v>
       </c>
     </row>
     <row r="7">
@@ -10504,7 +10429,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1537168</v>
+        <v>1530288</v>
       </c>
     </row>
   </sheetData>
@@ -16004,17 +15929,17 @@
         <v>0</v>
       </c>
       <c r="G134" s="6" t="n">
-        <v>6880</v>
+        <v>0</v>
       </c>
       <c r="H134" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I134" s="6" t="n">
-        <v>6880</v>
+        <v>0</v>
       </c>
       <c r="J134" s="5" t="inlineStr">
         <is>
-          <t>เก็บ 100% = 1 เรทเต็ม (รถ standby ระหว่างเที่ยว (เข้าต้นทาง 4.6 ชม. ไม่จบเที่ยว))</t>
+          <t>ไม่เก็บ [override: exclude_50] — โอสั่ง 4ส.ค.: วันนี้รถไปวิ่งงานแหลมฉบัง (บ้านบึง→WH-LCB TO-OTL17527 — คนละส่วนกับงาน บ้านบึง-P&amp;G) ไม่ใช่ standby รอ P&amp;G → ไม่เก็บ no_finish 100% (6,880)</t>
         </is>
       </c>
     </row>
@@ -30494,7 +30419,7 @@
         <v>1720</v>
       </c>
       <c r="X151" s="7" t="n">
-        <v>6880</v>
+        <v>0</v>
       </c>
       <c r="Y151" s="7" t="n">
         <v>0</v>
@@ -37037,7 +36962,7 @@
         <v>1720</v>
       </c>
       <c r="E151" s="7" t="n">
-        <v>6880</v>
+        <v>0</v>
       </c>
       <c r="F151" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Oatside July: restore 8001 26/7 standby charge per customer acceptance (grand back to 1,537,168)
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -33,8 +33,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Unmatched_Log'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Daily_Activity'!$A$1:$I$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Daily_Time_24h_Check'!$A$1:$M$143</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$142</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Plate_DestDay'!$A$1:$I$143</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Surcharge_50pct_1Trip'!$A$1:$L$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Manual_Extra_Trips'!$A$1:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Manual_Return_Trips'!$A$1:$D$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'NoWork_Outbound_50pct'!$A$1:$G$1</definedName>
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05 14:34</t>
+          <t>2026-08-07 15:55</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>193824</v>
+        <v>200704</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1530288</v>
+        <v>1537168</v>
       </c>
     </row>
   </sheetData>
@@ -802,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I142"/>
+  <dimension ref="A1:I143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
@@ -4706,22 +4706,22 @@
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E118" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F118" s="6" t="n">
-        <v>13760</v>
+        <v>0</v>
       </c>
       <c r="G118" s="6" t="n">
-        <v>0</v>
+        <v>6880</v>
       </c>
       <c r="H118" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I118" s="6" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
     </row>
     <row r="119">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -4739,31 +4739,31 @@
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E119" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F119" s="7" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G119" s="7" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H119" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I119" s="7" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="8" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
@@ -4784,10 +4784,10 @@
         <v>1720</v>
       </c>
       <c r="H120" s="6" t="n">
-        <v>3440</v>
+        <v>0</v>
       </c>
       <c r="I120" s="6" t="n">
-        <v>12040</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="121">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -4817,10 +4817,10 @@
         <v>1720</v>
       </c>
       <c r="H121" s="7" t="n">
-        <v>0</v>
+        <v>3440</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>8600</v>
+        <v>12040</v>
       </c>
     </row>
     <row r="122">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -4838,22 +4838,22 @@
         </is>
       </c>
       <c r="D122" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E122" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F122" s="6" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G122" s="6" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H122" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I122" s="6" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="123">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -4871,31 +4871,31 @@
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E123" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F123" s="7" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G123" s="7" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H123" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I123" s="7" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="n">
-        <v>46231</v>
+        <v>46230</v>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
@@ -4904,22 +4904,22 @@
         </is>
       </c>
       <c r="D124" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F124" s="6" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G124" s="6" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H124" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I124" s="6" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="125">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -5003,13 +5003,13 @@
         </is>
       </c>
       <c r="D127" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E127" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F127" s="7" t="n">
-        <v>20640</v>
+        <v>13760</v>
       </c>
       <c r="G127" s="7" t="n">
         <v>0</v>
@@ -5018,16 +5018,16 @@
         <v>0</v>
       </c>
       <c r="I127" s="7" t="n">
-        <v>20640</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="n">
-        <v>46232</v>
+        <v>46231</v>
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -5036,22 +5036,22 @@
         </is>
       </c>
       <c r="D128" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E128" s="6" t="n">
         <v>6880</v>
       </c>
       <c r="F128" s="6" t="n">
-        <v>6880</v>
+        <v>20640</v>
       </c>
       <c r="G128" s="6" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H128" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I128" s="6" t="n">
-        <v>8600</v>
+        <v>20640</v>
       </c>
     </row>
     <row r="129">
@@ -5060,7 +5060,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -5069,22 +5069,22 @@
         </is>
       </c>
       <c r="D129" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E129" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F129" s="7" t="n">
-        <v>13760</v>
+        <v>6880</v>
       </c>
       <c r="G129" s="7" t="n">
-        <v>0</v>
+        <v>1720</v>
       </c>
       <c r="H129" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I129" s="7" t="n">
-        <v>13760</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="130">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -5135,22 +5135,22 @@
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E131" s="7" t="n">
         <v>6880</v>
       </c>
       <c r="F131" s="7" t="n">
-        <v>6880</v>
+        <v>13760</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>1720</v>
+        <v>0</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I131" s="7" t="n">
-        <v>8600</v>
+        <v>13760</v>
       </c>
     </row>
     <row r="132">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
@@ -5188,11 +5188,11 @@
     </row>
     <row r="133">
       <c r="A133" s="9" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -5353,11 +5353,11 @@
     </row>
     <row r="138">
       <c r="A138" s="8" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -5411,10 +5411,10 @@
         <v>1720</v>
       </c>
       <c r="H139" s="7" t="n">
-        <v>3440</v>
+        <v>0</v>
       </c>
       <c r="I139" s="7" t="n">
-        <v>12040</v>
+        <v>8600</v>
       </c>
     </row>
     <row r="140">
@@ -5423,7 +5423,7 @@
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
@@ -5444,10 +5444,10 @@
         <v>1720</v>
       </c>
       <c r="H140" s="6" t="n">
-        <v>0</v>
+        <v>3440</v>
       </c>
       <c r="I140" s="6" t="n">
-        <v>8600</v>
+        <v>12040</v>
       </c>
     </row>
     <row r="141">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
@@ -5516,8 +5516,41 @@
         <v>8600</v>
       </c>
     </row>
+    <row r="143">
+      <c r="A143" s="9" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>BigC</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E143" s="7" t="n">
+        <v>6880</v>
+      </c>
+      <c r="F143" s="7" t="n">
+        <v>6880</v>
+      </c>
+      <c r="G143" s="7" t="n">
+        <v>1720</v>
+      </c>
+      <c r="H143" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" s="7" t="n">
+        <v>8600</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I142"/>
+  <autoFilter ref="A1:I143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5528,7 +5561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8821,7 +8854,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -8831,11 +8864,11 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>one_trip_billed_day</t>
+          <t>no_finish_day</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -8854,16 +8887,16 @@
         <v>6880</v>
       </c>
       <c r="L78" s="6" t="n">
-        <v>1720</v>
+        <v>6880</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
-        <v>46230</v>
+        <v>46229</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8888,7 +8921,7 @@
       <c r="H79" s="2" t="inlineStr"/>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
@@ -8905,7 +8938,7 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -8947,7 +8980,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -8985,11 +9018,11 @@
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>46232</v>
+        <v>46230</v>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
@@ -9014,7 +9047,7 @@
       <c r="H82" s="5" t="inlineStr"/>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr"/>
@@ -9031,7 +9064,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -9073,7 +9106,7 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -9111,11 +9144,11 @@
     </row>
     <row r="85">
       <c r="A85" s="9" t="n">
-        <v>46233</v>
+        <v>46232</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -9140,7 +9173,7 @@
       <c r="H85" s="2" t="inlineStr"/>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
@@ -9157,7 +9190,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -9199,7 +9232,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -9241,7 +9274,7 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -9283,7 +9316,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -9321,11 +9354,11 @@
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>71-5042</t>
+          <t>71-8009</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
@@ -9350,7 +9383,7 @@
       <c r="H90" s="5" t="inlineStr"/>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J90" s="5" t="inlineStr"/>
@@ -9367,7 +9400,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>71-8001</t>
+          <t>71-5042</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -9409,7 +9442,7 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>71-8002</t>
+          <t>71-8001</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
@@ -9451,7 +9484,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>71-8003</t>
+          <t>71-8002</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -9493,7 +9526,7 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>71-8009</t>
+          <t>71-8003</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -9529,8 +9562,50 @@
         <v>1720</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" s="9" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>71-8009</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>BigC</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>one_trip_billed_day</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="7" t="n">
+        <v>6880</v>
+      </c>
+      <c r="L95" s="7" t="n">
+        <v>1720</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L94"/>
+  <autoFilter ref="A1:L95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10399,7 +10474,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>193824</v>
+        <v>200704</v>
       </c>
     </row>
     <row r="7">
@@ -10429,7 +10504,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1530288</v>
+        <v>1537168</v>
       </c>
     </row>
   </sheetData>
@@ -15929,17 +16004,17 @@
         <v>0</v>
       </c>
       <c r="G134" s="6" t="n">
-        <v>0</v>
+        <v>6880</v>
       </c>
       <c r="H134" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I134" s="6" t="n">
-        <v>0</v>
+        <v>6880</v>
       </c>
       <c r="J134" s="5" t="inlineStr">
         <is>
-          <t>ไม่เก็บ [override: exclude_50] — โอสั่ง 4ส.ค.: วันนี้รถไปวิ่งงานแหลมฉบัง (บ้านบึง→WH-LCB TO-OTL17527 — คนละส่วนกับงาน บ้านบึง-P&amp;G) ไม่ใช่ standby รอ P&amp;G → ไม่เก็บ no_finish 100% (6,880)</t>
+          <t>เก็บ 100% = 1 เรทเต็ม (รถ standby ระหว่างเที่ยว (เข้าต้นทาง 4.6 ชม. ไม่จบเที่ยว))</t>
         </is>
       </c>
     </row>
@@ -30419,7 +30494,7 @@
         <v>1720</v>
       </c>
       <c r="X151" s="7" t="n">
-        <v>0</v>
+        <v>6880</v>
       </c>
       <c r="Y151" s="7" t="n">
         <v>0</v>
@@ -36962,7 +37037,7 @@
         <v>1720</v>
       </c>
       <c r="E151" s="7" t="n">
-        <v>0</v>
+        <v>6880</v>
       </c>
       <c r="F151" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Oatside July: fare by Origin-In fuel date per DHL agreement (grand 1,537,936, +768)
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 15:55</t>
+          <t>2026-08-09 10:57</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ก.ค. 2569: ฐาน 6,400 บาท (แถบน้ำมัน 31.00–31.99 บ./ล.) ปรับ +1.5% ต่อ 1 บาท (linear จากฐาน) อ้างอิงบางจาก ไฮดีเซล S (คอลัมน์ที่ 2) · ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% (ต่อเนื่องจาก 16/06/2569; รอทั้งวัน 100% คงเดิม)</t>
+          <t>ก.ค. 2569: ฐาน 6,400 บาท (แถบน้ำมัน 31.00–31.99 บ./ล.) ปรับ +1.5% ต่อ 1 บาท (linear จากฐาน) อ้างอิงบางจาก ไฮดีเซล S (คอลัมน์ที่ 2) · ราคาเที่ยวอิงราคาน้ำมัน ณ วันขึ้นของ (Origin In — ตกลงกับ DHL ส.ค. 2569) · ส่วนเพิ่มวันวิ่ง 1 เที่ยว 25% (ต่อเนื่องจาก 16/06/2569; รอทั้งวัน 100% คงเดิม)</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>1251712</v>
+        <v>1252480</v>
       </c>
     </row>
     <row r="14">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1537168</v>
+        <v>1537936</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +1874,7 @@
         <v>6688</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>1672</v>
@@ -1883,7 +1883,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>8360</v>
+        <v>8648</v>
       </c>
     </row>
     <row r="33">
@@ -1907,7 +1907,7 @@
         <v>6688</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>1672</v>
@@ -1916,7 +1916,7 @@
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>8360</v>
+        <v>8648</v>
       </c>
     </row>
     <row r="34">
@@ -1940,7 +1940,7 @@
         <v>6688</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="G34" s="6" t="n">
         <v>1672</v>
@@ -1949,7 +1949,7 @@
         <v>3344</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>11704</v>
+        <v>11992</v>
       </c>
     </row>
     <row r="35">
@@ -1973,7 +1973,7 @@
         <v>6688</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>1672</v>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>8360</v>
+        <v>8648</v>
       </c>
     </row>
     <row r="36">
@@ -4151,7 +4151,7 @@
         <v>6784</v>
       </c>
       <c r="F101" s="7" t="n">
-        <v>13568</v>
+        <v>13472</v>
       </c>
       <c r="G101" s="7" t="n">
         <v>0</v>
@@ -4160,7 +4160,7 @@
         <v>0</v>
       </c>
       <c r="I101" s="7" t="n">
-        <v>13568</v>
+        <v>13472</v>
       </c>
     </row>
     <row r="102">
@@ -4217,7 +4217,7 @@
         <v>6784</v>
       </c>
       <c r="F103" s="7" t="n">
-        <v>13568</v>
+        <v>13472</v>
       </c>
       <c r="G103" s="7" t="n">
         <v>0</v>
@@ -4226,7 +4226,7 @@
         <v>0</v>
       </c>
       <c r="I103" s="7" t="n">
-        <v>13568</v>
+        <v>13472</v>
       </c>
     </row>
     <row r="104">
@@ -4250,7 +4250,7 @@
         <v>6880</v>
       </c>
       <c r="F104" s="6" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="G104" s="6" t="n">
         <v>1720</v>
@@ -4259,7 +4259,7 @@
         <v>3440</v>
       </c>
       <c r="I104" s="6" t="n">
-        <v>12040</v>
+        <v>11944</v>
       </c>
     </row>
     <row r="105">
@@ -4283,7 +4283,7 @@
         <v>6880</v>
       </c>
       <c r="F105" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="G105" s="7" t="n">
         <v>1720</v>
@@ -4292,7 +4292,7 @@
         <v>0</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>8600</v>
+        <v>8504</v>
       </c>
     </row>
     <row r="106">
@@ -10414,7 +10414,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1251712</v>
+        <v>1252480</v>
       </c>
     </row>
     <row r="3">
@@ -10504,7 +10504,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1537168</v>
+        <v>1537936</v>
       </c>
     </row>
   </sheetData>
@@ -20800,7 +20800,7 @@
         <v>1</v>
       </c>
       <c r="V41" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="W41" s="7" t="n">
         <v>1672</v>
@@ -20888,7 +20888,7 @@
         <v>1</v>
       </c>
       <c r="V42" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="W42" s="6" t="n">
         <v>1672</v>
@@ -21064,7 +21064,7 @@
         <v>1</v>
       </c>
       <c r="V44" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="W44" s="6" t="n">
         <v>1672</v>
@@ -21152,7 +21152,7 @@
         <v>1</v>
       </c>
       <c r="V45" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="W45" s="7" t="n">
         <v>1672</v>
@@ -28548,7 +28548,7 @@
         <v>1</v>
       </c>
       <c r="V129" s="7" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="W129" s="7" t="n">
         <v>0</v>
@@ -28812,7 +28812,7 @@
         <v>1</v>
       </c>
       <c r="V132" s="6" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="W132" s="6" t="n">
         <v>0</v>
@@ -29076,7 +29076,7 @@
         <v>1</v>
       </c>
       <c r="V135" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="W135" s="7" t="n">
         <v>1720</v>
@@ -29428,7 +29428,7 @@
         <v>1</v>
       </c>
       <c r="V139" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="W139" s="7" t="n">
         <v>1720</v>
@@ -34281,7 +34281,7 @@
         </is>
       </c>
       <c r="C41" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>1672</v>
@@ -34306,7 +34306,7 @@
         </is>
       </c>
       <c r="C42" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="D42" s="6" t="n">
         <v>1672</v>
@@ -34356,7 +34356,7 @@
         </is>
       </c>
       <c r="C44" s="6" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="D44" s="6" t="n">
         <v>1672</v>
@@ -34381,7 +34381,7 @@
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>6688</v>
+        <v>6976</v>
       </c>
       <c r="D45" s="7" t="n">
         <v>1672</v>
@@ -36481,7 +36481,7 @@
         </is>
       </c>
       <c r="C129" s="7" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="D129" s="7" t="n">
         <v>0</v>
@@ -36556,7 +36556,7 @@
         </is>
       </c>
       <c r="C132" s="6" t="n">
-        <v>6784</v>
+        <v>6688</v>
       </c>
       <c r="D132" s="6" t="n">
         <v>0</v>
@@ -36631,7 +36631,7 @@
         </is>
       </c>
       <c r="C135" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="D135" s="7" t="n">
         <v>1720</v>
@@ -36731,7 +36731,7 @@
         </is>
       </c>
       <c r="C139" s="7" t="n">
-        <v>6880</v>
+        <v>6784</v>
       </c>
       <c r="D139" s="7" t="n">
         <v>1720</v>

</xml_diff>

<commit_message>
Oatside July: one-trip 25% follows trip fare (origin-date pricing) - grand 1,538,176
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
+++ b/reports/oatside-pg-2026/exports/00_Full_Workbook.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09 10:57</t>
+          <t>2026-08-09 11:52</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>200704</v>
+        <v>200944</v>
       </c>
     </row>
     <row r="21">
@@ -788,7 +788,7 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>1537936</v>
+        <v>1538176</v>
       </c>
     </row>
   </sheetData>
@@ -1877,13 +1877,13 @@
         <v>6976</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H32" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>8648</v>
+        <v>8720</v>
       </c>
     </row>
     <row r="33">
@@ -1910,13 +1910,13 @@
         <v>6976</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H33" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>8648</v>
+        <v>8720</v>
       </c>
     </row>
     <row r="34">
@@ -1943,13 +1943,13 @@
         <v>6976</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H34" s="6" t="n">
         <v>3344</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>11992</v>
+        <v>12064</v>
       </c>
     </row>
     <row r="35">
@@ -1976,13 +1976,13 @@
         <v>6976</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H35" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>8648</v>
+        <v>8720</v>
       </c>
     </row>
     <row r="36">
@@ -4253,13 +4253,13 @@
         <v>6784</v>
       </c>
       <c r="G104" s="6" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="H104" s="6" t="n">
         <v>3440</v>
       </c>
       <c r="I104" s="6" t="n">
-        <v>11944</v>
+        <v>11920</v>
       </c>
     </row>
     <row r="105">
@@ -4286,13 +4286,13 @@
         <v>6784</v>
       </c>
       <c r="G105" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="H105" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I105" s="7" t="n">
-        <v>8504</v>
+        <v>8480</v>
       </c>
     </row>
     <row r="106">
@@ -6485,7 +6485,7 @@
         <v>6688</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="22">
@@ -6527,7 +6527,7 @@
         <v>6688</v>
       </c>
       <c r="L22" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="23">
@@ -6569,7 +6569,7 @@
         <v>6688</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="24">
@@ -6611,7 +6611,7 @@
         <v>6688</v>
       </c>
       <c r="L24" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="25">
@@ -8341,7 +8341,7 @@
         <v>6880</v>
       </c>
       <c r="L65" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="66">
@@ -8383,7 +8383,7 @@
         <v>6880</v>
       </c>
       <c r="L66" s="6" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="67">
@@ -10474,7 +10474,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>200704</v>
+        <v>200944</v>
       </c>
     </row>
     <row r="7">
@@ -10504,7 +10504,7 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1537936</v>
+        <v>1538176</v>
       </c>
     </row>
   </sheetData>
@@ -12356,13 +12356,13 @@
         <v>6688</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H38" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>8360</v>
+        <v>8432</v>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
@@ -12394,13 +12394,13 @@
         <v>6688</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H39" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>8360</v>
+        <v>8432</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
@@ -12432,13 +12432,13 @@
         <v>6688</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H40" s="6" t="n">
         <v>3344</v>
       </c>
       <c r="I40" s="6" t="n">
-        <v>11704</v>
+        <v>11776</v>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
@@ -12470,13 +12470,13 @@
         <v>6688</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="H41" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>8360</v>
+        <v>8432</v>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
@@ -15396,13 +15396,13 @@
         <v>6880</v>
       </c>
       <c r="G118" s="6" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="H118" s="6" t="n">
         <v>3440</v>
       </c>
       <c r="I118" s="6" t="n">
-        <v>12040</v>
+        <v>12016</v>
       </c>
       <c r="J118" s="5" t="inlineStr">
         <is>
@@ -15510,13 +15510,13 @@
         <v>6880</v>
       </c>
       <c r="G121" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="H121" s="7" t="n">
         <v>0</v>
       </c>
       <c r="I121" s="7" t="n">
-        <v>8600</v>
+        <v>8576</v>
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
@@ -20803,7 +20803,7 @@
         <v>6976</v>
       </c>
       <c r="W41" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="X41" s="7" t="n">
         <v>0</v>
@@ -20891,7 +20891,7 @@
         <v>6976</v>
       </c>
       <c r="W42" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="X42" s="6" t="n">
         <v>0</v>
@@ -21067,7 +21067,7 @@
         <v>6976</v>
       </c>
       <c r="W44" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="X44" s="6" t="n">
         <v>0</v>
@@ -21155,7 +21155,7 @@
         <v>6976</v>
       </c>
       <c r="W45" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="X45" s="7" t="n">
         <v>0</v>
@@ -29079,7 +29079,7 @@
         <v>6784</v>
       </c>
       <c r="W135" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="X135" s="7" t="n">
         <v>0</v>
@@ -29431,7 +29431,7 @@
         <v>6784</v>
       </c>
       <c r="W139" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="X139" s="7" t="n">
         <v>0</v>
@@ -34284,7 +34284,7 @@
         <v>6976</v>
       </c>
       <c r="D41" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="E41" s="7" t="n">
         <v>0</v>
@@ -34309,7 +34309,7 @@
         <v>6976</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="E42" s="6" t="n">
         <v>0</v>
@@ -34359,7 +34359,7 @@
         <v>6976</v>
       </c>
       <c r="D44" s="6" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="E44" s="6" t="n">
         <v>0</v>
@@ -34384,7 +34384,7 @@
         <v>6976</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>1672</v>
+        <v>1744</v>
       </c>
       <c r="E45" s="7" t="n">
         <v>0</v>
@@ -36634,7 +36634,7 @@
         <v>6784</v>
       </c>
       <c r="D135" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="E135" s="7" t="n">
         <v>0</v>
@@ -36734,7 +36734,7 @@
         <v>6784</v>
       </c>
       <c r="D139" s="7" t="n">
-        <v>1720</v>
+        <v>1696</v>
       </c>
       <c r="E139" s="7" t="n">
         <v>0</v>

</xml_diff>